<commit_message>
ADD: new prices from 23.03.2026
</commit_message>
<xml_diff>
--- a/important_information/gta_eko_card.xlsx
+++ b/important_information/gta_eko_card.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sveto\OneDrive\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sveto\OneDrive\Desktop\eko_inv\important_information\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A522BE8D-A8C9-4CA8-BCBB-B725038C0A68}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7368D6BB-3957-4315-A75E-29167B7A5604}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{16EAB02D-4AF0-4E84-A118-5ED9D2D845E0}"/>
   </bookViews>
@@ -2848,13 +2848,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="14" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="49" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3194,7 +3196,7 @@
   <cols>
     <col min="1" max="1" width="27.85546875" style="2" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="12.140625" style="2" customWidth="1"/>
-    <col min="3" max="3" width="21.140625" style="2" customWidth="1"/>
+    <col min="3" max="3" width="21.140625" style="5" customWidth="1"/>
     <col min="4" max="4" width="14.5703125" style="2" customWidth="1"/>
     <col min="5" max="5" width="27.85546875" style="2" bestFit="1" customWidth="1"/>
     <col min="6" max="16384" width="10.85546875" style="2"/>
@@ -3207,7 +3209,7 @@
       <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="4" t="s">
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
@@ -3224,7 +3226,7 @@
       <c r="B2" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" s="5" t="s">
         <v>7</v>
       </c>
       <c r="D2" s="3">
@@ -3241,7 +3243,7 @@
       <c r="B3" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="C3" s="5" t="s">
         <v>9</v>
       </c>
       <c r="D3" s="3">
@@ -3258,7 +3260,7 @@
       <c r="B4" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="C4" s="5" t="s">
         <v>11</v>
       </c>
       <c r="D4" s="3">
@@ -3275,7 +3277,7 @@
       <c r="B5" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C5" s="2" t="s">
+      <c r="C5" s="5" t="s">
         <v>13</v>
       </c>
       <c r="D5" s="3">
@@ -3292,7 +3294,7 @@
       <c r="B6" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C6" s="2" t="s">
+      <c r="C6" s="5" t="s">
         <v>15</v>
       </c>
       <c r="D6" s="3">
@@ -3309,7 +3311,7 @@
       <c r="B7" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C7" s="2" t="s">
+      <c r="C7" s="5" t="s">
         <v>17</v>
       </c>
       <c r="D7" s="3">
@@ -3326,7 +3328,7 @@
       <c r="B8" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C8" s="2" t="s">
+      <c r="C8" s="5" t="s">
         <v>19</v>
       </c>
       <c r="D8" s="3">
@@ -3343,7 +3345,7 @@
       <c r="B9" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C9" s="2" t="s">
+      <c r="C9" s="5" t="s">
         <v>21</v>
       </c>
       <c r="D9" s="3">
@@ -3360,7 +3362,7 @@
       <c r="B10" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C10" s="2" t="s">
+      <c r="C10" s="5" t="s">
         <v>23</v>
       </c>
       <c r="D10" s="3">
@@ -3377,7 +3379,7 @@
       <c r="B11" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C11" s="2" t="s">
+      <c r="C11" s="5" t="s">
         <v>25</v>
       </c>
       <c r="D11" s="3">
@@ -3394,7 +3396,7 @@
       <c r="B12" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C12" s="2" t="s">
+      <c r="C12" s="5" t="s">
         <v>27</v>
       </c>
       <c r="D12" s="3">
@@ -3411,7 +3413,7 @@
       <c r="B13" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C13" s="2" t="s">
+      <c r="C13" s="5" t="s">
         <v>29</v>
       </c>
       <c r="D13" s="3">
@@ -3428,7 +3430,7 @@
       <c r="B14" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C14" s="2" t="s">
+      <c r="C14" s="5" t="s">
         <v>31</v>
       </c>
       <c r="D14" s="3">
@@ -3445,7 +3447,7 @@
       <c r="B15" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C15" s="2" t="s">
+      <c r="C15" s="5" t="s">
         <v>33</v>
       </c>
       <c r="D15" s="3">
@@ -3462,7 +3464,7 @@
       <c r="B16" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C16" s="2" t="s">
+      <c r="C16" s="5" t="s">
         <v>35</v>
       </c>
       <c r="D16" s="3">
@@ -3479,7 +3481,7 @@
       <c r="B17" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C17" s="2" t="s">
+      <c r="C17" s="5" t="s">
         <v>37</v>
       </c>
       <c r="D17" s="3">
@@ -3496,7 +3498,7 @@
       <c r="B18" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C18" s="2" t="s">
+      <c r="C18" s="5" t="s">
         <v>39</v>
       </c>
       <c r="D18" s="3">
@@ -3513,7 +3515,7 @@
       <c r="B19" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C19" s="2" t="s">
+      <c r="C19" s="5" t="s">
         <v>41</v>
       </c>
       <c r="D19" s="3">
@@ -3530,7 +3532,7 @@
       <c r="B20" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C20" s="2" t="s">
+      <c r="C20" s="5" t="s">
         <v>43</v>
       </c>
       <c r="D20" s="3">
@@ -3547,7 +3549,7 @@
       <c r="B21" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C21" s="2" t="s">
+      <c r="C21" s="5" t="s">
         <v>45</v>
       </c>
       <c r="D21" s="3">
@@ -3564,7 +3566,7 @@
       <c r="B22" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="C22" s="2" t="s">
+      <c r="C22" s="5" t="s">
         <v>48</v>
       </c>
       <c r="D22" s="3">
@@ -3581,7 +3583,7 @@
       <c r="B23" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="C23" s="2" t="s">
+      <c r="C23" s="5" t="s">
         <v>50</v>
       </c>
       <c r="D23" s="3">
@@ -3598,7 +3600,7 @@
       <c r="B24" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="C24" s="2" t="s">
+      <c r="C24" s="5" t="s">
         <v>52</v>
       </c>
       <c r="D24" s="3">
@@ -3615,7 +3617,7 @@
       <c r="B25" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="C25" s="2" t="s">
+      <c r="C25" s="5" t="s">
         <v>54</v>
       </c>
       <c r="D25" s="3">
@@ -3632,7 +3634,7 @@
       <c r="B26" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="C26" s="2" t="s">
+      <c r="C26" s="5" t="s">
         <v>56</v>
       </c>
       <c r="D26" s="3">
@@ -3649,7 +3651,7 @@
       <c r="B27" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="C27" s="2" t="s">
+      <c r="C27" s="5" t="s">
         <v>59</v>
       </c>
       <c r="D27" s="3">
@@ -3666,7 +3668,7 @@
       <c r="B28" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="C28" s="2" t="s">
+      <c r="C28" s="5" t="s">
         <v>61</v>
       </c>
       <c r="D28" s="3">
@@ -3683,7 +3685,7 @@
       <c r="B29" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="C29" s="2" t="s">
+      <c r="C29" s="5" t="s">
         <v>63</v>
       </c>
       <c r="D29" s="3">
@@ -3700,7 +3702,7 @@
       <c r="B30" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="C30" s="2" t="s">
+      <c r="C30" s="5" t="s">
         <v>65</v>
       </c>
       <c r="D30" s="3">
@@ -3717,7 +3719,7 @@
       <c r="B31" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="C31" s="2" t="s">
+      <c r="C31" s="5" t="s">
         <v>66</v>
       </c>
       <c r="D31" s="3">
@@ -3734,7 +3736,7 @@
       <c r="B32" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="C32" s="2" t="s">
+      <c r="C32" s="5" t="s">
         <v>67</v>
       </c>
       <c r="D32" s="3">
@@ -3751,7 +3753,7 @@
       <c r="B33" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="C33" s="2" t="s">
+      <c r="C33" s="5" t="s">
         <v>69</v>
       </c>
       <c r="D33" s="3">
@@ -3768,7 +3770,7 @@
       <c r="B34" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="C34" s="2" t="s">
+      <c r="C34" s="5" t="s">
         <v>71</v>
       </c>
       <c r="D34" s="3">
@@ -3785,7 +3787,7 @@
       <c r="B35" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="C35" s="2" t="s">
+      <c r="C35" s="5" t="s">
         <v>73</v>
       </c>
       <c r="D35" s="3">
@@ -3802,7 +3804,7 @@
       <c r="B36" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="C36" s="2" t="s">
+      <c r="C36" s="5" t="s">
         <v>75</v>
       </c>
       <c r="D36" s="3">
@@ -3819,7 +3821,7 @@
       <c r="B37" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="C37" s="2" t="s">
+      <c r="C37" s="5" t="s">
         <v>76</v>
       </c>
       <c r="D37" s="3">
@@ -3836,7 +3838,7 @@
       <c r="B38" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="C38" s="2" t="s">
+      <c r="C38" s="5" t="s">
         <v>78</v>
       </c>
       <c r="D38" s="3">
@@ -3853,7 +3855,7 @@
       <c r="B39" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="C39" s="2" t="s">
+      <c r="C39" s="5" t="s">
         <v>80</v>
       </c>
       <c r="D39" s="3">
@@ -3870,7 +3872,7 @@
       <c r="B40" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="C40" s="2" t="s">
+      <c r="C40" s="5" t="s">
         <v>82</v>
       </c>
       <c r="D40" s="3">
@@ -3887,7 +3889,7 @@
       <c r="B41" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="C41" s="2" t="s">
+      <c r="C41" s="5" t="s">
         <v>84</v>
       </c>
       <c r="D41" s="3">
@@ -3904,7 +3906,7 @@
       <c r="B42" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="C42" s="2" t="s">
+      <c r="C42" s="5" t="s">
         <v>86</v>
       </c>
       <c r="D42" s="3">
@@ -3921,7 +3923,7 @@
       <c r="B43" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="C43" s="2" t="s">
+      <c r="C43" s="5" t="s">
         <v>88</v>
       </c>
       <c r="D43" s="3">
@@ -3938,7 +3940,7 @@
       <c r="B44" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="C44" s="2" t="s">
+      <c r="C44" s="5" t="s">
         <v>90</v>
       </c>
       <c r="D44" s="3">
@@ -3955,7 +3957,7 @@
       <c r="B45" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="C45" s="2" t="s">
+      <c r="C45" s="5" t="s">
         <v>92</v>
       </c>
       <c r="D45" s="3">
@@ -3972,7 +3974,7 @@
       <c r="B46" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="C46" s="2" t="s">
+      <c r="C46" s="5" t="s">
         <v>94</v>
       </c>
       <c r="D46" s="3">
@@ -3989,7 +3991,7 @@
       <c r="B47" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="C47" s="2" t="s">
+      <c r="C47" s="5" t="s">
         <v>96</v>
       </c>
       <c r="D47" s="3">
@@ -4006,7 +4008,7 @@
       <c r="B48" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="C48" s="2" t="s">
+      <c r="C48" s="5" t="s">
         <v>98</v>
       </c>
       <c r="D48" s="3">
@@ -4023,7 +4025,7 @@
       <c r="B49" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="C49" s="2" t="s">
+      <c r="C49" s="5" t="s">
         <v>100</v>
       </c>
       <c r="D49" s="3">
@@ -4040,7 +4042,7 @@
       <c r="B50" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="C50" s="2" t="s">
+      <c r="C50" s="5" t="s">
         <v>102</v>
       </c>
       <c r="D50" s="3">
@@ -4057,7 +4059,7 @@
       <c r="B51" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="C51" s="2" t="s">
+      <c r="C51" s="5" t="s">
         <v>104</v>
       </c>
       <c r="D51" s="3">
@@ -4074,7 +4076,7 @@
       <c r="B52" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="C52" s="2" t="s">
+      <c r="C52" s="5" t="s">
         <v>106</v>
       </c>
       <c r="D52" s="3">
@@ -4091,7 +4093,7 @@
       <c r="B53" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="C53" s="2" t="s">
+      <c r="C53" s="5" t="s">
         <v>108</v>
       </c>
       <c r="D53" s="3">
@@ -4108,7 +4110,7 @@
       <c r="B54" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="C54" s="2" t="s">
+      <c r="C54" s="5" t="s">
         <v>110</v>
       </c>
       <c r="D54" s="3">
@@ -4125,7 +4127,7 @@
       <c r="B55" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="C55" s="2" t="s">
+      <c r="C55" s="5" t="s">
         <v>111</v>
       </c>
       <c r="D55" s="3">
@@ -4142,7 +4144,7 @@
       <c r="B56" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="C56" s="2" t="s">
+      <c r="C56" s="5" t="s">
         <v>113</v>
       </c>
       <c r="D56" s="3">
@@ -4159,7 +4161,7 @@
       <c r="B57" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="C57" s="2" t="s">
+      <c r="C57" s="5" t="s">
         <v>115</v>
       </c>
       <c r="D57" s="3">
@@ -4176,7 +4178,7 @@
       <c r="B58" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="C58" s="2" t="s">
+      <c r="C58" s="5" t="s">
         <v>117</v>
       </c>
       <c r="D58" s="3">
@@ -4193,7 +4195,7 @@
       <c r="B59" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="C59" s="2" t="s">
+      <c r="C59" s="5" t="s">
         <v>119</v>
       </c>
       <c r="D59" s="3">
@@ -4210,7 +4212,7 @@
       <c r="B60" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="C60" s="2" t="s">
+      <c r="C60" s="5" t="s">
         <v>121</v>
       </c>
       <c r="D60" s="3">
@@ -4227,7 +4229,7 @@
       <c r="B61" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="C61" s="2" t="s">
+      <c r="C61" s="5" t="s">
         <v>123</v>
       </c>
       <c r="D61" s="3">
@@ -4244,7 +4246,7 @@
       <c r="B62" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="C62" s="2" t="s">
+      <c r="C62" s="5" t="s">
         <v>125</v>
       </c>
       <c r="D62" s="3">
@@ -4261,7 +4263,7 @@
       <c r="B63" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="C63" s="2" t="s">
+      <c r="C63" s="5" t="s">
         <v>127</v>
       </c>
       <c r="D63" s="3">
@@ -4278,7 +4280,7 @@
       <c r="B64" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="C64" s="2" t="s">
+      <c r="C64" s="5" t="s">
         <v>129</v>
       </c>
       <c r="D64" s="3">
@@ -4295,7 +4297,7 @@
       <c r="B65" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="C65" s="2" t="s">
+      <c r="C65" s="5" t="s">
         <v>131</v>
       </c>
       <c r="D65" s="3">
@@ -4312,7 +4314,7 @@
       <c r="B66" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="C66" s="2" t="s">
+      <c r="C66" s="5" t="s">
         <v>133</v>
       </c>
       <c r="D66" s="3">
@@ -4329,7 +4331,7 @@
       <c r="B67" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="C67" s="2" t="s">
+      <c r="C67" s="5" t="s">
         <v>135</v>
       </c>
       <c r="D67" s="3">
@@ -4346,7 +4348,7 @@
       <c r="B68" s="2" t="s">
         <v>137</v>
       </c>
-      <c r="C68" s="2" t="s">
+      <c r="C68" s="5" t="s">
         <v>138</v>
       </c>
       <c r="D68" s="3">
@@ -4363,7 +4365,7 @@
       <c r="B69" s="2" t="s">
         <v>137</v>
       </c>
-      <c r="C69" s="2" t="s">
+      <c r="C69" s="5" t="s">
         <v>140</v>
       </c>
       <c r="D69" s="3">
@@ -4380,7 +4382,7 @@
       <c r="B70" s="2" t="s">
         <v>137</v>
       </c>
-      <c r="C70" s="2" t="s">
+      <c r="C70" s="5" t="s">
         <v>142</v>
       </c>
       <c r="D70" s="3">
@@ -4397,7 +4399,7 @@
       <c r="B71" s="2" t="s">
         <v>137</v>
       </c>
-      <c r="C71" s="2" t="s">
+      <c r="C71" s="5" t="s">
         <v>144</v>
       </c>
       <c r="D71" s="3">
@@ -4414,7 +4416,7 @@
       <c r="B72" s="2" t="s">
         <v>137</v>
       </c>
-      <c r="C72" s="2" t="s">
+      <c r="C72" s="5" t="s">
         <v>146</v>
       </c>
       <c r="D72" s="3">
@@ -4431,7 +4433,7 @@
       <c r="B73" s="2" t="s">
         <v>137</v>
       </c>
-      <c r="C73" s="2" t="s">
+      <c r="C73" s="5" t="s">
         <v>148</v>
       </c>
       <c r="D73" s="3">
@@ -4448,7 +4450,7 @@
       <c r="B74" s="2" t="s">
         <v>137</v>
       </c>
-      <c r="C74" s="2" t="s">
+      <c r="C74" s="5" t="s">
         <v>150</v>
       </c>
       <c r="D74" s="3">
@@ -4465,7 +4467,7 @@
       <c r="B75" s="2" t="s">
         <v>137</v>
       </c>
-      <c r="C75" s="2" t="s">
+      <c r="C75" s="5" t="s">
         <v>152</v>
       </c>
       <c r="D75" s="3">
@@ -4482,7 +4484,7 @@
       <c r="B76" s="2" t="s">
         <v>137</v>
       </c>
-      <c r="C76" s="2" t="s">
+      <c r="C76" s="5" t="s">
         <v>154</v>
       </c>
       <c r="D76" s="3">
@@ -4499,7 +4501,7 @@
       <c r="B77" s="2" t="s">
         <v>137</v>
       </c>
-      <c r="C77" s="2" t="s">
+      <c r="C77" s="5" t="s">
         <v>156</v>
       </c>
       <c r="D77" s="3">
@@ -4516,7 +4518,7 @@
       <c r="B78" s="2" t="s">
         <v>137</v>
       </c>
-      <c r="C78" s="2" t="s">
+      <c r="C78" s="5" t="s">
         <v>158</v>
       </c>
       <c r="D78" s="3">
@@ -4533,7 +4535,7 @@
       <c r="B79" s="2" t="s">
         <v>137</v>
       </c>
-      <c r="C79" s="2" t="s">
+      <c r="C79" s="5" t="s">
         <v>160</v>
       </c>
       <c r="D79" s="3">
@@ -4550,7 +4552,7 @@
       <c r="B80" s="2" t="s">
         <v>137</v>
       </c>
-      <c r="C80" s="2" t="s">
+      <c r="C80" s="5" t="s">
         <v>162</v>
       </c>
       <c r="D80" s="3">
@@ -4567,7 +4569,7 @@
       <c r="B81" s="2" t="s">
         <v>137</v>
       </c>
-      <c r="C81" s="2" t="s">
+      <c r="C81" s="5" t="s">
         <v>164</v>
       </c>
       <c r="D81" s="3">
@@ -4584,7 +4586,7 @@
       <c r="B82" s="2" t="s">
         <v>137</v>
       </c>
-      <c r="C82" s="2" t="s">
+      <c r="C82" s="5" t="s">
         <v>166</v>
       </c>
       <c r="D82" s="3">
@@ -4601,7 +4603,7 @@
       <c r="B83" s="2" t="s">
         <v>137</v>
       </c>
-      <c r="C83" s="2" t="s">
+      <c r="C83" s="5" t="s">
         <v>168</v>
       </c>
       <c r="D83" s="3">
@@ -4618,7 +4620,7 @@
       <c r="B84" s="2" t="s">
         <v>137</v>
       </c>
-      <c r="C84" s="2" t="s">
+      <c r="C84" s="5" t="s">
         <v>170</v>
       </c>
       <c r="D84" s="3">
@@ -4635,7 +4637,7 @@
       <c r="B85" s="2" t="s">
         <v>137</v>
       </c>
-      <c r="C85" s="2" t="s">
+      <c r="C85" s="5" t="s">
         <v>171</v>
       </c>
       <c r="D85" s="3">
@@ -4652,7 +4654,7 @@
       <c r="B86" s="2" t="s">
         <v>137</v>
       </c>
-      <c r="C86" s="2" t="s">
+      <c r="C86" s="5" t="s">
         <v>172</v>
       </c>
       <c r="D86" s="3">
@@ -4669,7 +4671,7 @@
       <c r="B87" s="2" t="s">
         <v>137</v>
       </c>
-      <c r="C87" s="2" t="s">
+      <c r="C87" s="5" t="s">
         <v>174</v>
       </c>
       <c r="D87" s="3">
@@ -4686,7 +4688,7 @@
       <c r="B88" s="2" t="s">
         <v>137</v>
       </c>
-      <c r="C88" s="2" t="s">
+      <c r="C88" s="5" t="s">
         <v>176</v>
       </c>
       <c r="D88" s="3">
@@ -4703,7 +4705,7 @@
       <c r="B89" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="C89" s="2" t="s">
+      <c r="C89" s="5" t="s">
         <v>178</v>
       </c>
       <c r="D89" s="3">
@@ -4720,7 +4722,7 @@
       <c r="B90" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="C90" s="2" t="s">
+      <c r="C90" s="5" t="s">
         <v>180</v>
       </c>
       <c r="D90" s="3">
@@ -4737,7 +4739,7 @@
       <c r="B91" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="C91" s="2" t="s">
+      <c r="C91" s="5" t="s">
         <v>182</v>
       </c>
       <c r="D91" s="3">
@@ -4754,7 +4756,7 @@
       <c r="B92" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="C92" s="2" t="s">
+      <c r="C92" s="5" t="s">
         <v>184</v>
       </c>
       <c r="D92" s="3">
@@ -4771,7 +4773,7 @@
       <c r="B93" s="2" t="s">
         <v>137</v>
       </c>
-      <c r="C93" s="2" t="s">
+      <c r="C93" s="5" t="s">
         <v>185</v>
       </c>
       <c r="D93" s="3">
@@ -4788,7 +4790,7 @@
       <c r="B94" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="C94" s="2" t="s">
+      <c r="C94" s="5" t="s">
         <v>187</v>
       </c>
       <c r="D94" s="3">
@@ -4805,7 +4807,7 @@
       <c r="B95" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="C95" s="2" t="s">
+      <c r="C95" s="5" t="s">
         <v>188</v>
       </c>
       <c r="D95" s="3">
@@ -4822,7 +4824,7 @@
       <c r="B96" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="C96" s="2" t="s">
+      <c r="C96" s="5" t="s">
         <v>189</v>
       </c>
       <c r="D96" s="3">
@@ -4839,7 +4841,7 @@
       <c r="B97" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="C97" s="2" t="s">
+      <c r="C97" s="5" t="s">
         <v>191</v>
       </c>
       <c r="D97" s="3">
@@ -4856,7 +4858,7 @@
       <c r="B98" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="C98" s="2" t="s">
+      <c r="C98" s="5" t="s">
         <v>193</v>
       </c>
       <c r="D98" s="3">
@@ -4873,7 +4875,7 @@
       <c r="B99" s="2" t="s">
         <v>195</v>
       </c>
-      <c r="C99" s="2" t="s">
+      <c r="C99" s="5" t="s">
         <v>196</v>
       </c>
       <c r="D99" s="3">
@@ -4890,7 +4892,7 @@
       <c r="B100" s="2" t="s">
         <v>195</v>
       </c>
-      <c r="C100" s="2" t="s">
+      <c r="C100" s="5" t="s">
         <v>198</v>
       </c>
       <c r="D100" s="3">
@@ -4907,7 +4909,7 @@
       <c r="B101" s="2" t="s">
         <v>195</v>
       </c>
-      <c r="C101" s="2" t="s">
+      <c r="C101" s="5" t="s">
         <v>200</v>
       </c>
       <c r="D101" s="3">
@@ -4924,7 +4926,7 @@
       <c r="B102" s="2" t="s">
         <v>195</v>
       </c>
-      <c r="C102" s="2" t="s">
+      <c r="C102" s="5" t="s">
         <v>202</v>
       </c>
       <c r="D102" s="3">
@@ -4941,7 +4943,7 @@
       <c r="B103" s="2" t="s">
         <v>195</v>
       </c>
-      <c r="C103" s="2" t="s">
+      <c r="C103" s="5" t="s">
         <v>204</v>
       </c>
       <c r="D103" s="3">
@@ -4958,7 +4960,7 @@
       <c r="B104" s="2" t="s">
         <v>195</v>
       </c>
-      <c r="C104" s="2" t="s">
+      <c r="C104" s="5" t="s">
         <v>206</v>
       </c>
       <c r="D104" s="3">
@@ -4975,7 +4977,7 @@
       <c r="B105" s="2" t="s">
         <v>195</v>
       </c>
-      <c r="C105" s="2" t="s">
+      <c r="C105" s="5" t="s">
         <v>208</v>
       </c>
       <c r="D105" s="3">
@@ -4992,7 +4994,7 @@
       <c r="B106" s="2" t="s">
         <v>195</v>
       </c>
-      <c r="C106" s="2" t="s">
+      <c r="C106" s="5" t="s">
         <v>210</v>
       </c>
       <c r="D106" s="3">
@@ -5009,7 +5011,7 @@
       <c r="B107" s="2" t="s">
         <v>195</v>
       </c>
-      <c r="C107" s="2" t="s">
+      <c r="C107" s="5" t="s">
         <v>212</v>
       </c>
       <c r="D107" s="3">
@@ -5026,7 +5028,7 @@
       <c r="B108" s="2" t="s">
         <v>195</v>
       </c>
-      <c r="C108" s="2" t="s">
+      <c r="C108" s="5" t="s">
         <v>214</v>
       </c>
       <c r="D108" s="3">
@@ -5043,7 +5045,7 @@
       <c r="B109" s="2" t="s">
         <v>195</v>
       </c>
-      <c r="C109" s="2" t="s">
+      <c r="C109" s="5" t="s">
         <v>216</v>
       </c>
       <c r="D109" s="3">
@@ -5060,7 +5062,7 @@
       <c r="B110" s="2" t="s">
         <v>195</v>
       </c>
-      <c r="C110" s="2" t="s">
+      <c r="C110" s="5" t="s">
         <v>218</v>
       </c>
       <c r="D110" s="3">
@@ -5077,7 +5079,7 @@
       <c r="B111" s="2" t="s">
         <v>195</v>
       </c>
-      <c r="C111" s="2" t="s">
+      <c r="C111" s="5" t="s">
         <v>220</v>
       </c>
       <c r="D111" s="3">
@@ -5094,7 +5096,7 @@
       <c r="B112" s="2" t="s">
         <v>195</v>
       </c>
-      <c r="C112" s="2" t="s">
+      <c r="C112" s="5" t="s">
         <v>222</v>
       </c>
       <c r="D112" s="3">
@@ -5111,7 +5113,7 @@
       <c r="B113" s="2" t="s">
         <v>195</v>
       </c>
-      <c r="C113" s="2" t="s">
+      <c r="C113" s="5" t="s">
         <v>224</v>
       </c>
       <c r="D113" s="3">
@@ -5128,7 +5130,7 @@
       <c r="B114" s="2" t="s">
         <v>195</v>
       </c>
-      <c r="C114" s="2" t="s">
+      <c r="C114" s="5" t="s">
         <v>226</v>
       </c>
       <c r="D114" s="3">
@@ -5145,7 +5147,7 @@
       <c r="B115" s="2" t="s">
         <v>195</v>
       </c>
-      <c r="C115" s="2" t="s">
+      <c r="C115" s="5" t="s">
         <v>228</v>
       </c>
       <c r="D115" s="3">
@@ -5162,7 +5164,7 @@
       <c r="B116" s="2" t="s">
         <v>195</v>
       </c>
-      <c r="C116" s="2" t="s">
+      <c r="C116" s="5" t="s">
         <v>230</v>
       </c>
       <c r="D116" s="3">
@@ -5179,7 +5181,7 @@
       <c r="B117" s="2" t="s">
         <v>195</v>
       </c>
-      <c r="C117" s="2" t="s">
+      <c r="C117" s="5" t="s">
         <v>232</v>
       </c>
       <c r="D117" s="3">
@@ -5196,7 +5198,7 @@
       <c r="B118" s="2" t="s">
         <v>195</v>
       </c>
-      <c r="C118" s="2" t="s">
+      <c r="C118" s="5" t="s">
         <v>234</v>
       </c>
       <c r="D118" s="3">
@@ -5213,7 +5215,7 @@
       <c r="B119" s="2" t="s">
         <v>195</v>
       </c>
-      <c r="C119" s="2" t="s">
+      <c r="C119" s="5" t="s">
         <v>236</v>
       </c>
       <c r="D119" s="3">
@@ -5230,7 +5232,7 @@
       <c r="B120" s="2" t="s">
         <v>195</v>
       </c>
-      <c r="C120" s="2" t="s">
+      <c r="C120" s="5" t="s">
         <v>238</v>
       </c>
       <c r="D120" s="3">
@@ -5247,7 +5249,7 @@
       <c r="B121" s="2" t="s">
         <v>195</v>
       </c>
-      <c r="C121" s="2" t="s">
+      <c r="C121" s="5" t="s">
         <v>240</v>
       </c>
       <c r="D121" s="3">
@@ -5264,7 +5266,7 @@
       <c r="B122" s="2" t="s">
         <v>195</v>
       </c>
-      <c r="C122" s="2" t="s">
+      <c r="C122" s="5" t="s">
         <v>242</v>
       </c>
       <c r="D122" s="3">
@@ -5281,7 +5283,7 @@
       <c r="B123" s="2" t="s">
         <v>195</v>
       </c>
-      <c r="C123" s="2" t="s">
+      <c r="C123" s="5" t="s">
         <v>244</v>
       </c>
       <c r="D123" s="3">
@@ -5298,7 +5300,7 @@
       <c r="B124" s="2" t="s">
         <v>195</v>
       </c>
-      <c r="C124" s="2" t="s">
+      <c r="C124" s="5" t="s">
         <v>246</v>
       </c>
       <c r="D124" s="3">
@@ -5315,7 +5317,7 @@
       <c r="B125" s="2" t="s">
         <v>195</v>
       </c>
-      <c r="C125" s="2" t="s">
+      <c r="C125" s="5" t="s">
         <v>248</v>
       </c>
       <c r="D125" s="3">
@@ -5332,7 +5334,7 @@
       <c r="B126" s="2" t="s">
         <v>195</v>
       </c>
-      <c r="C126" s="2" t="s">
+      <c r="C126" s="5" t="s">
         <v>250</v>
       </c>
       <c r="D126" s="3">
@@ -5349,7 +5351,7 @@
       <c r="B127" s="2" t="s">
         <v>195</v>
       </c>
-      <c r="C127" s="2" t="s">
+      <c r="C127" s="5" t="s">
         <v>252</v>
       </c>
       <c r="D127" s="3">
@@ -5366,7 +5368,7 @@
       <c r="B128" s="2" t="s">
         <v>195</v>
       </c>
-      <c r="C128" s="2" t="s">
+      <c r="C128" s="5" t="s">
         <v>254</v>
       </c>
       <c r="D128" s="3">
@@ -5383,7 +5385,7 @@
       <c r="B129" s="2" t="s">
         <v>195</v>
       </c>
-      <c r="C129" s="2" t="s">
+      <c r="C129" s="5" t="s">
         <v>256</v>
       </c>
       <c r="D129" s="3">
@@ -5400,7 +5402,7 @@
       <c r="B130" s="2" t="s">
         <v>195</v>
       </c>
-      <c r="C130" s="2" t="s">
+      <c r="C130" s="5" t="s">
         <v>258</v>
       </c>
       <c r="D130" s="3">
@@ -5417,7 +5419,7 @@
       <c r="B131" s="2" t="s">
         <v>195</v>
       </c>
-      <c r="C131" s="2" t="s">
+      <c r="C131" s="5" t="s">
         <v>260</v>
       </c>
       <c r="D131" s="3">
@@ -5434,7 +5436,7 @@
       <c r="B132" s="2" t="s">
         <v>195</v>
       </c>
-      <c r="C132" s="2" t="s">
+      <c r="C132" s="5" t="s">
         <v>262</v>
       </c>
       <c r="D132" s="3">
@@ -5451,7 +5453,7 @@
       <c r="B133" s="2" t="s">
         <v>195</v>
       </c>
-      <c r="C133" s="2" t="s">
+      <c r="C133" s="5" t="s">
         <v>264</v>
       </c>
       <c r="D133" s="3">
@@ -5468,7 +5470,7 @@
       <c r="B134" s="2" t="s">
         <v>195</v>
       </c>
-      <c r="C134" s="2" t="s">
+      <c r="C134" s="5" t="s">
         <v>266</v>
       </c>
       <c r="D134" s="3">
@@ -5485,7 +5487,7 @@
       <c r="B135" s="2" t="s">
         <v>195</v>
       </c>
-      <c r="C135" s="2" t="s">
+      <c r="C135" s="5" t="s">
         <v>268</v>
       </c>
       <c r="D135" s="3">
@@ -5502,7 +5504,7 @@
       <c r="B136" s="2" t="s">
         <v>195</v>
       </c>
-      <c r="C136" s="2" t="s">
+      <c r="C136" s="5" t="s">
         <v>270</v>
       </c>
       <c r="D136" s="3">
@@ -5519,7 +5521,7 @@
       <c r="B137" s="2" t="s">
         <v>195</v>
       </c>
-      <c r="C137" s="2" t="s">
+      <c r="C137" s="5" t="s">
         <v>272</v>
       </c>
       <c r="D137" s="3">
@@ -5536,7 +5538,7 @@
       <c r="B138" s="2" t="s">
         <v>195</v>
       </c>
-      <c r="C138" s="2" t="s">
+      <c r="C138" s="5" t="s">
         <v>274</v>
       </c>
       <c r="D138" s="3">
@@ -5553,7 +5555,7 @@
       <c r="B139" s="2" t="s">
         <v>195</v>
       </c>
-      <c r="C139" s="2" t="s">
+      <c r="C139" s="5" t="s">
         <v>276</v>
       </c>
       <c r="D139" s="3">
@@ -5570,7 +5572,7 @@
       <c r="B140" s="2" t="s">
         <v>195</v>
       </c>
-      <c r="C140" s="2" t="s">
+      <c r="C140" s="5" t="s">
         <v>278</v>
       </c>
       <c r="D140" s="3">
@@ -5587,7 +5589,7 @@
       <c r="B141" s="2" t="s">
         <v>195</v>
       </c>
-      <c r="C141" s="2" t="s">
+      <c r="C141" s="5" t="s">
         <v>280</v>
       </c>
       <c r="D141" s="3">
@@ -5604,7 +5606,7 @@
       <c r="B142" s="2" t="s">
         <v>195</v>
       </c>
-      <c r="C142" s="2" t="s">
+      <c r="C142" s="5" t="s">
         <v>282</v>
       </c>
       <c r="D142" s="3">
@@ -5621,7 +5623,7 @@
       <c r="B143" s="2" t="s">
         <v>195</v>
       </c>
-      <c r="C143" s="2" t="s">
+      <c r="C143" s="5" t="s">
         <v>284</v>
       </c>
       <c r="D143" s="3">
@@ -5638,7 +5640,7 @@
       <c r="B144" s="2" t="s">
         <v>195</v>
       </c>
-      <c r="C144" s="2" t="s">
+      <c r="C144" s="5" t="s">
         <v>286</v>
       </c>
       <c r="D144" s="3">
@@ -5655,7 +5657,7 @@
       <c r="B145" s="2" t="s">
         <v>195</v>
       </c>
-      <c r="C145" s="2" t="s">
+      <c r="C145" s="5" t="s">
         <v>288</v>
       </c>
       <c r="D145" s="3">
@@ -5672,7 +5674,7 @@
       <c r="B146" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="C146" s="2" t="s">
+      <c r="C146" s="5" t="s">
         <v>290</v>
       </c>
       <c r="D146" s="3">
@@ -5689,7 +5691,7 @@
       <c r="B147" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="C147" s="2" t="s">
+      <c r="C147" s="5" t="s">
         <v>292</v>
       </c>
       <c r="D147" s="3">
@@ -5706,7 +5708,7 @@
       <c r="B148" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="C148" s="2" t="s">
+      <c r="C148" s="5" t="s">
         <v>294</v>
       </c>
       <c r="D148" s="3">
@@ -5723,7 +5725,7 @@
       <c r="B149" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="C149" s="2" t="s">
+      <c r="C149" s="5" t="s">
         <v>296</v>
       </c>
       <c r="D149" s="3">
@@ -5740,7 +5742,7 @@
       <c r="B150" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="C150" s="2" t="s">
+      <c r="C150" s="5" t="s">
         <v>298</v>
       </c>
       <c r="D150" s="3">
@@ -5757,7 +5759,7 @@
       <c r="B151" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="C151" s="2" t="s">
+      <c r="C151" s="5" t="s">
         <v>300</v>
       </c>
       <c r="D151" s="3">
@@ -5774,7 +5776,7 @@
       <c r="B152" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="C152" s="2" t="s">
+      <c r="C152" s="5" t="s">
         <v>302</v>
       </c>
       <c r="D152" s="3">
@@ -5791,7 +5793,7 @@
       <c r="B153" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="C153" s="2" t="s">
+      <c r="C153" s="5" t="s">
         <v>303</v>
       </c>
       <c r="D153" s="3">
@@ -5808,7 +5810,7 @@
       <c r="B154" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="C154" s="2" t="s">
+      <c r="C154" s="5" t="s">
         <v>304</v>
       </c>
       <c r="D154" s="3">
@@ -5825,7 +5827,7 @@
       <c r="B155" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="C155" s="2" t="s">
+      <c r="C155" s="5" t="s">
         <v>305</v>
       </c>
       <c r="D155" s="3">
@@ -5842,7 +5844,7 @@
       <c r="B156" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="C156" s="2" t="s">
+      <c r="C156" s="5" t="s">
         <v>306</v>
       </c>
       <c r="D156" s="3">
@@ -5859,7 +5861,7 @@
       <c r="B157" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="C157" s="2" t="s">
+      <c r="C157" s="5" t="s">
         <v>307</v>
       </c>
       <c r="D157" s="3">
@@ -5876,7 +5878,7 @@
       <c r="B158" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="C158" s="2" t="s">
+      <c r="C158" s="5" t="s">
         <v>308</v>
       </c>
       <c r="D158" s="3">
@@ -5893,7 +5895,7 @@
       <c r="B159" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="C159" s="2" t="s">
+      <c r="C159" s="5" t="s">
         <v>310</v>
       </c>
       <c r="D159" s="3">
@@ -5910,7 +5912,7 @@
       <c r="B160" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="C160" s="2" t="s">
+      <c r="C160" s="5" t="s">
         <v>312</v>
       </c>
       <c r="D160" s="3">
@@ -5927,7 +5929,7 @@
       <c r="B161" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="C161" s="2" t="s">
+      <c r="C161" s="5" t="s">
         <v>314</v>
       </c>
       <c r="D161" s="3">
@@ -5944,7 +5946,7 @@
       <c r="B162" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="C162" s="2" t="s">
+      <c r="C162" s="5" t="s">
         <v>316</v>
       </c>
       <c r="D162" s="3">
@@ -5961,7 +5963,7 @@
       <c r="B163" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="C163" s="2" t="s">
+      <c r="C163" s="5" t="s">
         <v>318</v>
       </c>
       <c r="D163" s="3">
@@ -5978,7 +5980,7 @@
       <c r="B164" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="C164" s="2" t="s">
+      <c r="C164" s="5" t="s">
         <v>320</v>
       </c>
       <c r="D164" s="3">
@@ -5995,7 +5997,7 @@
       <c r="B165" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="C165" s="2" t="s">
+      <c r="C165" s="5" t="s">
         <v>322</v>
       </c>
       <c r="D165" s="3">
@@ -6012,7 +6014,7 @@
       <c r="B166" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="C166" s="2" t="s">
+      <c r="C166" s="5" t="s">
         <v>324</v>
       </c>
       <c r="D166" s="3">
@@ -6029,7 +6031,7 @@
       <c r="B167" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="C167" s="2" t="s">
+      <c r="C167" s="5" t="s">
         <v>326</v>
       </c>
       <c r="D167" s="3">
@@ -6046,7 +6048,7 @@
       <c r="B168" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="C168" s="2" t="s">
+      <c r="C168" s="5" t="s">
         <v>328</v>
       </c>
       <c r="D168" s="3">
@@ -6063,7 +6065,7 @@
       <c r="B169" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="C169" s="2" t="s">
+      <c r="C169" s="5" t="s">
         <v>330</v>
       </c>
       <c r="D169" s="3">
@@ -6080,7 +6082,7 @@
       <c r="B170" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="C170" s="2" t="s">
+      <c r="C170" s="5" t="s">
         <v>332</v>
       </c>
       <c r="D170" s="3">
@@ -6097,7 +6099,7 @@
       <c r="B171" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="C171" s="2" t="s">
+      <c r="C171" s="5" t="s">
         <v>334</v>
       </c>
       <c r="D171" s="3">
@@ -6114,7 +6116,7 @@
       <c r="B172" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="C172" s="2" t="s">
+      <c r="C172" s="5" t="s">
         <v>336</v>
       </c>
       <c r="D172" s="3">
@@ -6131,7 +6133,7 @@
       <c r="B173" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="C173" s="2" t="s">
+      <c r="C173" s="5" t="s">
         <v>338</v>
       </c>
       <c r="D173" s="3">
@@ -6148,7 +6150,7 @@
       <c r="B174" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="C174" s="2" t="s">
+      <c r="C174" s="5" t="s">
         <v>340</v>
       </c>
       <c r="D174" s="3">
@@ -6165,7 +6167,7 @@
       <c r="B175" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="C175" s="2" t="s">
+      <c r="C175" s="5" t="s">
         <v>342</v>
       </c>
       <c r="D175" s="3">
@@ -6182,7 +6184,7 @@
       <c r="B176" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="C176" s="2" t="s">
+      <c r="C176" s="5" t="s">
         <v>344</v>
       </c>
       <c r="D176" s="3">
@@ -6199,7 +6201,7 @@
       <c r="B177" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="C177" s="2" t="s">
+      <c r="C177" s="5" t="s">
         <v>346</v>
       </c>
       <c r="D177" s="3">
@@ -6216,7 +6218,7 @@
       <c r="B178" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="C178" s="2" t="s">
+      <c r="C178" s="5" t="s">
         <v>348</v>
       </c>
       <c r="D178" s="3">
@@ -6233,7 +6235,7 @@
       <c r="B179" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="C179" s="2" t="s">
+      <c r="C179" s="5" t="s">
         <v>350</v>
       </c>
       <c r="D179" s="3">
@@ -6250,7 +6252,7 @@
       <c r="B180" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="C180" s="2" t="s">
+      <c r="C180" s="5" t="s">
         <v>352</v>
       </c>
       <c r="D180" s="3">
@@ -6267,7 +6269,7 @@
       <c r="B181" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="C181" s="2" t="s">
+      <c r="C181" s="5" t="s">
         <v>354</v>
       </c>
       <c r="D181" s="3">
@@ -6284,7 +6286,7 @@
       <c r="B182" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="C182" s="2" t="s">
+      <c r="C182" s="5" t="s">
         <v>356</v>
       </c>
       <c r="D182" s="3">
@@ -6301,7 +6303,7 @@
       <c r="B183" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="C183" s="2" t="s">
+      <c r="C183" s="5" t="s">
         <v>358</v>
       </c>
       <c r="D183" s="3">
@@ -6318,7 +6320,7 @@
       <c r="B184" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="C184" s="2" t="s">
+      <c r="C184" s="5" t="s">
         <v>360</v>
       </c>
       <c r="D184" s="3">
@@ -6335,7 +6337,7 @@
       <c r="B185" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="C185" s="2" t="s">
+      <c r="C185" s="5" t="s">
         <v>362</v>
       </c>
       <c r="D185" s="3">
@@ -6352,7 +6354,7 @@
       <c r="B186" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="C186" s="2" t="s">
+      <c r="C186" s="5" t="s">
         <v>364</v>
       </c>
       <c r="D186" s="3">
@@ -6369,7 +6371,7 @@
       <c r="B187" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="C187" s="2" t="s">
+      <c r="C187" s="5" t="s">
         <v>366</v>
       </c>
       <c r="D187" s="3">
@@ -6386,7 +6388,7 @@
       <c r="B188" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="C188" s="2" t="s">
+      <c r="C188" s="5" t="s">
         <v>368</v>
       </c>
       <c r="D188" s="3">
@@ -6403,7 +6405,7 @@
       <c r="B189" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="C189" s="2" t="s">
+      <c r="C189" s="5" t="s">
         <v>370</v>
       </c>
       <c r="D189" s="3">
@@ -6420,7 +6422,7 @@
       <c r="B190" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="C190" s="2" t="s">
+      <c r="C190" s="5" t="s">
         <v>372</v>
       </c>
       <c r="D190" s="3">
@@ -6437,7 +6439,7 @@
       <c r="B191" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="C191" s="2" t="s">
+      <c r="C191" s="5" t="s">
         <v>374</v>
       </c>
       <c r="D191" s="3">
@@ -6454,7 +6456,7 @@
       <c r="B192" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="C192" s="2" t="s">
+      <c r="C192" s="5" t="s">
         <v>376</v>
       </c>
       <c r="D192" s="3">
@@ -6471,7 +6473,7 @@
       <c r="B193" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="C193" s="2" t="s">
+      <c r="C193" s="5" t="s">
         <v>378</v>
       </c>
       <c r="D193" s="3">
@@ -6488,7 +6490,7 @@
       <c r="B194" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="C194" s="2" t="s">
+      <c r="C194" s="5" t="s">
         <v>380</v>
       </c>
       <c r="D194" s="3">
@@ -6505,7 +6507,7 @@
       <c r="B195" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="C195" s="2" t="s">
+      <c r="C195" s="5" t="s">
         <v>382</v>
       </c>
       <c r="D195" s="3">
@@ -6522,7 +6524,7 @@
       <c r="B196" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="C196" s="2" t="s">
+      <c r="C196" s="5" t="s">
         <v>384</v>
       </c>
       <c r="D196" s="3">
@@ -6539,7 +6541,7 @@
       <c r="B197" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="C197" s="2" t="s">
+      <c r="C197" s="5" t="s">
         <v>386</v>
       </c>
       <c r="D197" s="3">
@@ -6556,7 +6558,7 @@
       <c r="B198" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="C198" s="2" t="s">
+      <c r="C198" s="5" t="s">
         <v>388</v>
       </c>
       <c r="D198" s="3">
@@ -6573,7 +6575,7 @@
       <c r="B199" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="C199" s="2" t="s">
+      <c r="C199" s="5" t="s">
         <v>390</v>
       </c>
       <c r="D199" s="3">
@@ -6590,7 +6592,7 @@
       <c r="B200" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="C200" s="2" t="s">
+      <c r="C200" s="5" t="s">
         <v>392</v>
       </c>
       <c r="D200" s="3">
@@ -6607,7 +6609,7 @@
       <c r="B201" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="C201" s="2" t="s">
+      <c r="C201" s="5" t="s">
         <v>394</v>
       </c>
       <c r="D201" s="3">
@@ -6624,7 +6626,7 @@
       <c r="B202" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="C202" s="2" t="s">
+      <c r="C202" s="5" t="s">
         <v>396</v>
       </c>
       <c r="D202" s="3">
@@ -6641,7 +6643,7 @@
       <c r="B203" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="C203" s="2" t="s">
+      <c r="C203" s="5" t="s">
         <v>398</v>
       </c>
       <c r="D203" s="3">
@@ -6658,7 +6660,7 @@
       <c r="B204" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="C204" s="2" t="s">
+      <c r="C204" s="5" t="s">
         <v>400</v>
       </c>
       <c r="D204" s="3">
@@ -6675,7 +6677,7 @@
       <c r="B205" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="C205" s="2" t="s">
+      <c r="C205" s="5" t="s">
         <v>402</v>
       </c>
       <c r="D205" s="3">
@@ -6692,7 +6694,7 @@
       <c r="B206" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="C206" s="2" t="s">
+      <c r="C206" s="5" t="s">
         <v>404</v>
       </c>
       <c r="D206" s="3">
@@ -6709,7 +6711,7 @@
       <c r="B207" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="C207" s="2" t="s">
+      <c r="C207" s="5" t="s">
         <v>406</v>
       </c>
       <c r="D207" s="3">
@@ -6726,7 +6728,7 @@
       <c r="B208" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="C208" s="2" t="s">
+      <c r="C208" s="5" t="s">
         <v>408</v>
       </c>
       <c r="D208" s="3">
@@ -6743,7 +6745,7 @@
       <c r="B209" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="C209" s="2" t="s">
+      <c r="C209" s="5" t="s">
         <v>410</v>
       </c>
       <c r="D209" s="3">
@@ -6760,7 +6762,7 @@
       <c r="B210" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="C210" s="2" t="s">
+      <c r="C210" s="5" t="s">
         <v>412</v>
       </c>
       <c r="D210" s="3">
@@ -6777,7 +6779,7 @@
       <c r="B211" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="C211" s="2" t="s">
+      <c r="C211" s="5" t="s">
         <v>414</v>
       </c>
       <c r="D211" s="3">
@@ -6794,7 +6796,7 @@
       <c r="B212" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="C212" s="2" t="s">
+      <c r="C212" s="5" t="s">
         <v>416</v>
       </c>
       <c r="D212" s="3">
@@ -6811,7 +6813,7 @@
       <c r="B213" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="C213" s="2" t="s">
+      <c r="C213" s="5" t="s">
         <v>418</v>
       </c>
       <c r="D213" s="3">
@@ -6828,7 +6830,7 @@
       <c r="B214" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="C214" s="2" t="s">
+      <c r="C214" s="5" t="s">
         <v>420</v>
       </c>
       <c r="D214" s="3">
@@ -6845,7 +6847,7 @@
       <c r="B215" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="C215" s="2" t="s">
+      <c r="C215" s="5" t="s">
         <v>422</v>
       </c>
       <c r="D215" s="3">
@@ -6862,7 +6864,7 @@
       <c r="B216" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="C216" s="2" t="s">
+      <c r="C216" s="5" t="s">
         <v>424</v>
       </c>
       <c r="D216" s="3">
@@ -6879,7 +6881,7 @@
       <c r="B217" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="C217" s="2" t="s">
+      <c r="C217" s="5" t="s">
         <v>426</v>
       </c>
       <c r="D217" s="3">
@@ -6896,7 +6898,7 @@
       <c r="B218" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="C218" s="2" t="s">
+      <c r="C218" s="5" t="s">
         <v>428</v>
       </c>
       <c r="D218" s="3">
@@ -6913,7 +6915,7 @@
       <c r="B219" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="C219" s="2" t="s">
+      <c r="C219" s="5" t="s">
         <v>430</v>
       </c>
       <c r="D219" s="3">
@@ -6930,7 +6932,7 @@
       <c r="B220" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="C220" s="2" t="s">
+      <c r="C220" s="5" t="s">
         <v>432</v>
       </c>
       <c r="D220" s="3">
@@ -6947,7 +6949,7 @@
       <c r="B221" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="C221" s="2" t="s">
+      <c r="C221" s="5" t="s">
         <v>434</v>
       </c>
       <c r="D221" s="3">
@@ -6964,7 +6966,7 @@
       <c r="B222" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="C222" s="2" t="s">
+      <c r="C222" s="5" t="s">
         <v>436</v>
       </c>
       <c r="D222" s="3">
@@ -6981,7 +6983,7 @@
       <c r="B223" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="C223" s="2" t="s">
+      <c r="C223" s="5" t="s">
         <v>438</v>
       </c>
       <c r="D223" s="3">
@@ -6998,7 +7000,7 @@
       <c r="B224" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="C224" s="2" t="s">
+      <c r="C224" s="5" t="s">
         <v>440</v>
       </c>
       <c r="D224" s="3">
@@ -7015,7 +7017,7 @@
       <c r="B225" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="C225" s="2" t="s">
+      <c r="C225" s="5" t="s">
         <v>442</v>
       </c>
       <c r="D225" s="3">
@@ -7032,7 +7034,7 @@
       <c r="B226" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="C226" s="2" t="s">
+      <c r="C226" s="5" t="s">
         <v>444</v>
       </c>
       <c r="D226" s="3">
@@ -7049,7 +7051,7 @@
       <c r="B227" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="C227" s="2" t="s">
+      <c r="C227" s="5" t="s">
         <v>446</v>
       </c>
       <c r="D227" s="3">
@@ -7066,7 +7068,7 @@
       <c r="B228" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="C228" s="2" t="s">
+      <c r="C228" s="5" t="s">
         <v>448</v>
       </c>
       <c r="D228" s="3">
@@ -7083,7 +7085,7 @@
       <c r="B229" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="C229" s="2" t="s">
+      <c r="C229" s="5" t="s">
         <v>450</v>
       </c>
       <c r="D229" s="3">
@@ -7100,7 +7102,7 @@
       <c r="B230" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="C230" s="2" t="s">
+      <c r="C230" s="5" t="s">
         <v>452</v>
       </c>
       <c r="D230" s="3">
@@ -7117,7 +7119,7 @@
       <c r="B231" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="C231" s="2" t="s">
+      <c r="C231" s="5" t="s">
         <v>454</v>
       </c>
       <c r="D231" s="3">
@@ -7134,7 +7136,7 @@
       <c r="B232" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="C232" s="2" t="s">
+      <c r="C232" s="5" t="s">
         <v>456</v>
       </c>
       <c r="D232" s="3">
@@ -7151,7 +7153,7 @@
       <c r="B233" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="C233" s="2" t="s">
+      <c r="C233" s="5" t="s">
         <v>458</v>
       </c>
       <c r="D233" s="3">
@@ -7168,7 +7170,7 @@
       <c r="B234" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="C234" s="2" t="s">
+      <c r="C234" s="5" t="s">
         <v>460</v>
       </c>
       <c r="D234" s="3">
@@ -7185,7 +7187,7 @@
       <c r="B235" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="C235" s="2" t="s">
+      <c r="C235" s="5" t="s">
         <v>462</v>
       </c>
       <c r="D235" s="3">
@@ -7202,7 +7204,7 @@
       <c r="B236" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="C236" s="2" t="s">
+      <c r="C236" s="5" t="s">
         <v>464</v>
       </c>
       <c r="D236" s="3">
@@ -7219,7 +7221,7 @@
       <c r="B237" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="C237" s="2" t="s">
+      <c r="C237" s="5" t="s">
         <v>466</v>
       </c>
       <c r="D237" s="3">
@@ -7236,7 +7238,7 @@
       <c r="B238" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="C238" s="2" t="s">
+      <c r="C238" s="5" t="s">
         <v>468</v>
       </c>
       <c r="D238" s="3">
@@ -7253,7 +7255,7 @@
       <c r="B239" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="C239" s="2" t="s">
+      <c r="C239" s="5" t="s">
         <v>470</v>
       </c>
       <c r="D239" s="3">
@@ -7270,7 +7272,7 @@
       <c r="B240" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="C240" s="2" t="s">
+      <c r="C240" s="5" t="s">
         <v>472</v>
       </c>
       <c r="D240" s="3">
@@ -7287,7 +7289,7 @@
       <c r="B241" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="C241" s="2" t="s">
+      <c r="C241" s="5" t="s">
         <v>474</v>
       </c>
       <c r="D241" s="3">
@@ -7304,7 +7306,7 @@
       <c r="B242" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="C242" s="2" t="s">
+      <c r="C242" s="5" t="s">
         <v>476</v>
       </c>
       <c r="D242" s="3">
@@ -7321,7 +7323,7 @@
       <c r="B243" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="C243" s="2" t="s">
+      <c r="C243" s="5" t="s">
         <v>478</v>
       </c>
       <c r="D243" s="3">
@@ -7338,7 +7340,7 @@
       <c r="B244" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="C244" s="2" t="s">
+      <c r="C244" s="5" t="s">
         <v>480</v>
       </c>
       <c r="D244" s="3">
@@ -7355,7 +7357,7 @@
       <c r="B245" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="C245" s="2" t="s">
+      <c r="C245" s="5" t="s">
         <v>482</v>
       </c>
       <c r="D245" s="3">
@@ -7372,7 +7374,7 @@
       <c r="B246" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="C246" s="2" t="s">
+      <c r="C246" s="5" t="s">
         <v>484</v>
       </c>
       <c r="D246" s="3">
@@ -7389,7 +7391,7 @@
       <c r="B247" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="C247" s="2" t="s">
+      <c r="C247" s="5" t="s">
         <v>486</v>
       </c>
       <c r="D247" s="3">
@@ -7406,7 +7408,7 @@
       <c r="B248" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="C248" s="2" t="s">
+      <c r="C248" s="5" t="s">
         <v>488</v>
       </c>
       <c r="D248" s="3">
@@ -7423,7 +7425,7 @@
       <c r="B249" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="C249" s="2" t="s">
+      <c r="C249" s="5" t="s">
         <v>490</v>
       </c>
       <c r="D249" s="3">
@@ -7440,7 +7442,7 @@
       <c r="B250" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="C250" s="2" t="s">
+      <c r="C250" s="5" t="s">
         <v>492</v>
       </c>
       <c r="D250" s="3">
@@ -7457,7 +7459,7 @@
       <c r="B251" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="C251" s="2" t="s">
+      <c r="C251" s="5" t="s">
         <v>494</v>
       </c>
       <c r="D251" s="3">
@@ -7474,7 +7476,7 @@
       <c r="B252" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="C252" s="2" t="s">
+      <c r="C252" s="5" t="s">
         <v>496</v>
       </c>
       <c r="D252" s="3">
@@ -7491,7 +7493,7 @@
       <c r="B253" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="C253" s="2" t="s">
+      <c r="C253" s="5" t="s">
         <v>498</v>
       </c>
       <c r="D253" s="3">
@@ -7508,7 +7510,7 @@
       <c r="B254" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="C254" s="2" t="s">
+      <c r="C254" s="5" t="s">
         <v>500</v>
       </c>
       <c r="D254" s="3">
@@ -7525,7 +7527,7 @@
       <c r="B255" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="C255" s="2" t="s">
+      <c r="C255" s="5" t="s">
         <v>502</v>
       </c>
       <c r="D255" s="3">
@@ -7542,7 +7544,7 @@
       <c r="B256" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="C256" s="2" t="s">
+      <c r="C256" s="5" t="s">
         <v>504</v>
       </c>
       <c r="D256" s="3">
@@ -7559,7 +7561,7 @@
       <c r="B257" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="C257" s="2" t="s">
+      <c r="C257" s="5" t="s">
         <v>506</v>
       </c>
       <c r="D257" s="3">
@@ -7576,7 +7578,7 @@
       <c r="B258" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="C258" s="2" t="s">
+      <c r="C258" s="5" t="s">
         <v>508</v>
       </c>
       <c r="D258" s="3">
@@ -7593,7 +7595,7 @@
       <c r="B259" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="C259" s="2" t="s">
+      <c r="C259" s="5" t="s">
         <v>510</v>
       </c>
       <c r="D259" s="3">
@@ -7610,7 +7612,7 @@
       <c r="B260" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="C260" s="2" t="s">
+      <c r="C260" s="5" t="s">
         <v>512</v>
       </c>
       <c r="D260" s="3">
@@ -7627,7 +7629,7 @@
       <c r="B261" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="C261" s="2" t="s">
+      <c r="C261" s="5" t="s">
         <v>514</v>
       </c>
       <c r="D261" s="3">
@@ -7644,7 +7646,7 @@
       <c r="B262" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="C262" s="2" t="s">
+      <c r="C262" s="5" t="s">
         <v>516</v>
       </c>
       <c r="D262" s="3">
@@ -7661,7 +7663,7 @@
       <c r="B263" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="C263" s="2" t="s">
+      <c r="C263" s="5" t="s">
         <v>518</v>
       </c>
       <c r="D263" s="3">
@@ -7678,7 +7680,7 @@
       <c r="B264" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="C264" s="2" t="s">
+      <c r="C264" s="5" t="s">
         <v>520</v>
       </c>
       <c r="D264" s="3">
@@ -7695,7 +7697,7 @@
       <c r="B265" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="C265" s="2" t="s">
+      <c r="C265" s="5" t="s">
         <v>522</v>
       </c>
       <c r="D265" s="3">
@@ -7712,7 +7714,7 @@
       <c r="B266" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="C266" s="2" t="s">
+      <c r="C266" s="5" t="s">
         <v>524</v>
       </c>
       <c r="D266" s="3">
@@ -7729,7 +7731,7 @@
       <c r="B267" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="C267" s="2" t="s">
+      <c r="C267" s="5" t="s">
         <v>526</v>
       </c>
       <c r="D267" s="3">
@@ -7746,7 +7748,7 @@
       <c r="B268" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="C268" s="2" t="s">
+      <c r="C268" s="5" t="s">
         <v>528</v>
       </c>
       <c r="D268" s="3">
@@ -7763,7 +7765,7 @@
       <c r="B269" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="C269" s="2" t="s">
+      <c r="C269" s="5" t="s">
         <v>530</v>
       </c>
       <c r="D269" s="3">
@@ -7780,7 +7782,7 @@
       <c r="B270" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="C270" s="2" t="s">
+      <c r="C270" s="5" t="s">
         <v>532</v>
       </c>
       <c r="D270" s="3">
@@ -7797,7 +7799,7 @@
       <c r="B271" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="C271" s="2" t="s">
+      <c r="C271" s="5" t="s">
         <v>534</v>
       </c>
       <c r="D271" s="3">
@@ -7814,7 +7816,7 @@
       <c r="B272" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="C272" s="2" t="s">
+      <c r="C272" s="5" t="s">
         <v>536</v>
       </c>
       <c r="D272" s="3">
@@ -7831,7 +7833,7 @@
       <c r="B273" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C273" s="2" t="s">
+      <c r="C273" s="5" t="s">
         <v>538</v>
       </c>
       <c r="D273" s="3">
@@ -7848,7 +7850,7 @@
       <c r="B274" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C274" s="2" t="s">
+      <c r="C274" s="5" t="s">
         <v>539</v>
       </c>
       <c r="D274" s="3">
@@ -7865,7 +7867,7 @@
       <c r="B275" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C275" s="2" t="s">
+      <c r="C275" s="5" t="s">
         <v>540</v>
       </c>
       <c r="D275" s="3">
@@ -7882,7 +7884,7 @@
       <c r="B276" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C276" s="2" t="s">
+      <c r="C276" s="5" t="s">
         <v>541</v>
       </c>
       <c r="D276" s="3">
@@ -7899,7 +7901,7 @@
       <c r="B277" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C277" s="2" t="s">
+      <c r="C277" s="5" t="s">
         <v>543</v>
       </c>
       <c r="D277" s="3">
@@ -7916,7 +7918,7 @@
       <c r="B278" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C278" s="2" t="s">
+      <c r="C278" s="5" t="s">
         <v>545</v>
       </c>
       <c r="D278" s="3">
@@ -7933,7 +7935,7 @@
       <c r="B279" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C279" s="2" t="s">
+      <c r="C279" s="5" t="s">
         <v>547</v>
       </c>
       <c r="D279" s="3">
@@ -7950,7 +7952,7 @@
       <c r="B280" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C280" s="2" t="s">
+      <c r="C280" s="5" t="s">
         <v>549</v>
       </c>
       <c r="D280" s="3">
@@ -7967,7 +7969,7 @@
       <c r="B281" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C281" s="2" t="s">
+      <c r="C281" s="5" t="s">
         <v>551</v>
       </c>
       <c r="D281" s="3">
@@ -7984,7 +7986,7 @@
       <c r="B282" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C282" s="2" t="s">
+      <c r="C282" s="5" t="s">
         <v>553</v>
       </c>
       <c r="D282" s="3">
@@ -8001,7 +8003,7 @@
       <c r="B283" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C283" s="2" t="s">
+      <c r="C283" s="5" t="s">
         <v>555</v>
       </c>
       <c r="D283" s="3">
@@ -8018,7 +8020,7 @@
       <c r="B284" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C284" s="2" t="s">
+      <c r="C284" s="5" t="s">
         <v>557</v>
       </c>
       <c r="D284" s="3">
@@ -8035,7 +8037,7 @@
       <c r="B285" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C285" s="2" t="s">
+      <c r="C285" s="5" t="s">
         <v>559</v>
       </c>
       <c r="D285" s="3">
@@ -8052,7 +8054,7 @@
       <c r="B286" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C286" s="2" t="s">
+      <c r="C286" s="5" t="s">
         <v>561</v>
       </c>
       <c r="D286" s="3">
@@ -8069,7 +8071,7 @@
       <c r="B287" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C287" s="2" t="s">
+      <c r="C287" s="5" t="s">
         <v>563</v>
       </c>
       <c r="D287" s="3">
@@ -8086,7 +8088,7 @@
       <c r="B288" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C288" s="2" t="s">
+      <c r="C288" s="5" t="s">
         <v>565</v>
       </c>
       <c r="D288" s="3">
@@ -8103,7 +8105,7 @@
       <c r="B289" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C289" s="2" t="s">
+      <c r="C289" s="5" t="s">
         <v>567</v>
       </c>
       <c r="D289" s="3">
@@ -8120,7 +8122,7 @@
       <c r="B290" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C290" s="2" t="s">
+      <c r="C290" s="5" t="s">
         <v>569</v>
       </c>
       <c r="D290" s="3">
@@ -8137,7 +8139,7 @@
       <c r="B291" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C291" s="2" t="s">
+      <c r="C291" s="5" t="s">
         <v>571</v>
       </c>
       <c r="D291" s="3">
@@ -8154,7 +8156,7 @@
       <c r="B292" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C292" s="2" t="s">
+      <c r="C292" s="5" t="s">
         <v>573</v>
       </c>
       <c r="D292" s="3">
@@ -8171,7 +8173,7 @@
       <c r="B293" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="C293" s="2" t="s">
+      <c r="C293" s="5" t="s">
         <v>575</v>
       </c>
       <c r="D293" s="3">
@@ -8188,7 +8190,7 @@
       <c r="B294" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="C294" s="2" t="s">
+      <c r="C294" s="5" t="s">
         <v>577</v>
       </c>
       <c r="D294" s="3">
@@ -8205,7 +8207,7 @@
       <c r="B295" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="C295" s="2" t="s">
+      <c r="C295" s="5" t="s">
         <v>579</v>
       </c>
       <c r="D295" s="3">
@@ -8222,7 +8224,7 @@
       <c r="B296" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="C296" s="2" t="s">
+      <c r="C296" s="5" t="s">
         <v>581</v>
       </c>
       <c r="D296" s="3">
@@ -8239,7 +8241,7 @@
       <c r="B297" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="C297" s="2" t="s">
+      <c r="C297" s="5" t="s">
         <v>583</v>
       </c>
       <c r="D297" s="3">
@@ -8256,7 +8258,7 @@
       <c r="B298" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="C298" s="2" t="s">
+      <c r="C298" s="5" t="s">
         <v>585</v>
       </c>
       <c r="D298" s="3">
@@ -8273,7 +8275,7 @@
       <c r="B299" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="C299" s="2" t="s">
+      <c r="C299" s="5" t="s">
         <v>587</v>
       </c>
       <c r="D299" s="3">
@@ -8290,7 +8292,7 @@
       <c r="B300" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="C300" s="2" t="s">
+      <c r="C300" s="5" t="s">
         <v>589</v>
       </c>
       <c r="D300" s="3">
@@ -8307,7 +8309,7 @@
       <c r="B301" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="C301" s="2" t="s">
+      <c r="C301" s="5" t="s">
         <v>591</v>
       </c>
       <c r="D301" s="3">
@@ -8324,7 +8326,7 @@
       <c r="B302" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="C302" s="2" t="s">
+      <c r="C302" s="5" t="s">
         <v>593</v>
       </c>
       <c r="D302" s="3">
@@ -8341,7 +8343,7 @@
       <c r="B303" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="C303" s="2" t="s">
+      <c r="C303" s="5" t="s">
         <v>595</v>
       </c>
       <c r="D303" s="3">
@@ -8358,7 +8360,7 @@
       <c r="B304" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="C304" s="2" t="s">
+      <c r="C304" s="5" t="s">
         <v>597</v>
       </c>
       <c r="D304" s="3">
@@ -8375,7 +8377,7 @@
       <c r="B305" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="C305" s="2" t="s">
+      <c r="C305" s="5" t="s">
         <v>599</v>
       </c>
       <c r="D305" s="3">
@@ -8392,7 +8394,7 @@
       <c r="B306" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="C306" s="2" t="s">
+      <c r="C306" s="5" t="s">
         <v>601</v>
       </c>
       <c r="D306" s="3">
@@ -8409,7 +8411,7 @@
       <c r="B307" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="C307" s="2" t="s">
+      <c r="C307" s="5" t="s">
         <v>603</v>
       </c>
       <c r="D307" s="3">
@@ -8426,7 +8428,7 @@
       <c r="B308" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="C308" s="2" t="s">
+      <c r="C308" s="5" t="s">
         <v>605</v>
       </c>
       <c r="D308" s="3">
@@ -8443,7 +8445,7 @@
       <c r="B309" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="C309" s="2" t="s">
+      <c r="C309" s="5" t="s">
         <v>607</v>
       </c>
       <c r="D309" s="3">
@@ -8460,7 +8462,7 @@
       <c r="B310" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="C310" s="2" t="s">
+      <c r="C310" s="5" t="s">
         <v>609</v>
       </c>
       <c r="D310" s="3">
@@ -8477,7 +8479,7 @@
       <c r="B311" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="C311" s="2" t="s">
+      <c r="C311" s="5" t="s">
         <v>611</v>
       </c>
       <c r="D311" s="3">
@@ -8494,7 +8496,7 @@
       <c r="B312" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="C312" s="2" t="s">
+      <c r="C312" s="5" t="s">
         <v>613</v>
       </c>
       <c r="D312" s="3">
@@ -8511,7 +8513,7 @@
       <c r="B313" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="C313" s="2" t="s">
+      <c r="C313" s="5" t="s">
         <v>615</v>
       </c>
       <c r="D313" s="3">
@@ -8528,7 +8530,7 @@
       <c r="B314" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="C314" s="2" t="s">
+      <c r="C314" s="5" t="s">
         <v>617</v>
       </c>
       <c r="D314" s="3">
@@ -8545,7 +8547,7 @@
       <c r="B315" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="C315" s="2" t="s">
+      <c r="C315" s="5" t="s">
         <v>619</v>
       </c>
       <c r="D315" s="3">
@@ -8562,7 +8564,7 @@
       <c r="B316" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="C316" s="2" t="s">
+      <c r="C316" s="5" t="s">
         <v>621</v>
       </c>
       <c r="D316" s="3">
@@ -8579,7 +8581,7 @@
       <c r="B317" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="C317" s="2" t="s">
+      <c r="C317" s="5" t="s">
         <v>623</v>
       </c>
       <c r="D317" s="3">
@@ -8596,7 +8598,7 @@
       <c r="B318" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="C318" s="2" t="s">
+      <c r="C318" s="5" t="s">
         <v>625</v>
       </c>
       <c r="D318" s="3">
@@ -8613,7 +8615,7 @@
       <c r="B319" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="C319" s="2" t="s">
+      <c r="C319" s="5" t="s">
         <v>627</v>
       </c>
       <c r="D319" s="3">
@@ -8630,7 +8632,7 @@
       <c r="B320" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="C320" s="2" t="s">
+      <c r="C320" s="5" t="s">
         <v>629</v>
       </c>
       <c r="D320" s="3">
@@ -8647,7 +8649,7 @@
       <c r="B321" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="C321" s="2" t="s">
+      <c r="C321" s="5" t="s">
         <v>631</v>
       </c>
       <c r="D321" s="3">
@@ -8664,7 +8666,7 @@
       <c r="B322" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="C322" s="2" t="s">
+      <c r="C322" s="5" t="s">
         <v>633</v>
       </c>
       <c r="D322" s="3">
@@ -8681,7 +8683,7 @@
       <c r="B323" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="C323" s="2" t="s">
+      <c r="C323" s="5" t="s">
         <v>635</v>
       </c>
       <c r="D323" s="3">
@@ -8698,7 +8700,7 @@
       <c r="B324" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="C324" s="2" t="s">
+      <c r="C324" s="5" t="s">
         <v>637</v>
       </c>
       <c r="D324" s="3">
@@ -8715,7 +8717,7 @@
       <c r="B325" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="C325" s="2" t="s">
+      <c r="C325" s="5" t="s">
         <v>639</v>
       </c>
       <c r="D325" s="3">
@@ -8732,7 +8734,7 @@
       <c r="B326" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="C326" s="2" t="s">
+      <c r="C326" s="5" t="s">
         <v>641</v>
       </c>
       <c r="D326" s="3">
@@ -8749,7 +8751,7 @@
       <c r="B327" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="C327" s="2" t="s">
+      <c r="C327" s="5" t="s">
         <v>643</v>
       </c>
       <c r="D327" s="3">
@@ -8766,7 +8768,7 @@
       <c r="B328" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="C328" s="2" t="s">
+      <c r="C328" s="5" t="s">
         <v>645</v>
       </c>
       <c r="D328" s="3">
@@ -8783,7 +8785,7 @@
       <c r="B329" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="C329" s="2" t="s">
+      <c r="C329" s="5" t="s">
         <v>647</v>
       </c>
       <c r="D329" s="3">
@@ -8800,7 +8802,7 @@
       <c r="B330" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="C330" s="2" t="s">
+      <c r="C330" s="5" t="s">
         <v>649</v>
       </c>
       <c r="D330" s="3">
@@ -8817,7 +8819,7 @@
       <c r="B331" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="C331" s="2" t="s">
+      <c r="C331" s="5" t="s">
         <v>651</v>
       </c>
       <c r="D331" s="3">
@@ -8834,7 +8836,7 @@
       <c r="B332" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="C332" s="2" t="s">
+      <c r="C332" s="5" t="s">
         <v>653</v>
       </c>
       <c r="D332" s="3">
@@ -8851,7 +8853,7 @@
       <c r="B333" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="C333" s="2" t="s">
+      <c r="C333" s="5" t="s">
         <v>655</v>
       </c>
       <c r="D333" s="3">
@@ -8868,7 +8870,7 @@
       <c r="B334" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="C334" s="2" t="s">
+      <c r="C334" s="5" t="s">
         <v>657</v>
       </c>
       <c r="D334" s="3">
@@ -8885,7 +8887,7 @@
       <c r="B335" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="C335" s="2" t="s">
+      <c r="C335" s="5" t="s">
         <v>659</v>
       </c>
       <c r="D335" s="3">
@@ -8902,7 +8904,7 @@
       <c r="B336" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="C336" s="2" t="s">
+      <c r="C336" s="5" t="s">
         <v>661</v>
       </c>
       <c r="D336" s="3">
@@ -8919,7 +8921,7 @@
       <c r="B337" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="C337" s="2" t="s">
+      <c r="C337" s="5" t="s">
         <v>663</v>
       </c>
       <c r="D337" s="3">
@@ -8936,7 +8938,7 @@
       <c r="B338" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="C338" s="2" t="s">
+      <c r="C338" s="5" t="s">
         <v>665</v>
       </c>
       <c r="D338" s="3">
@@ -8953,7 +8955,7 @@
       <c r="B339" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="C339" s="2" t="s">
+      <c r="C339" s="5" t="s">
         <v>667</v>
       </c>
       <c r="D339" s="3">
@@ -8970,7 +8972,7 @@
       <c r="B340" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="C340" s="2" t="s">
+      <c r="C340" s="5" t="s">
         <v>669</v>
       </c>
       <c r="D340" s="3">
@@ -8987,7 +8989,7 @@
       <c r="B341" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="C341" s="2" t="s">
+      <c r="C341" s="5" t="s">
         <v>671</v>
       </c>
       <c r="D341" s="3">
@@ -9004,7 +9006,7 @@
       <c r="B342" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="C342" s="2" t="s">
+      <c r="C342" s="5" t="s">
         <v>673</v>
       </c>
       <c r="D342" s="3">
@@ -9021,7 +9023,7 @@
       <c r="B343" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="C343" s="2" t="s">
+      <c r="C343" s="5" t="s">
         <v>675</v>
       </c>
       <c r="D343" s="3">
@@ -9038,7 +9040,7 @@
       <c r="B344" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="C344" s="2" t="s">
+      <c r="C344" s="5" t="s">
         <v>677</v>
       </c>
       <c r="D344" s="3">
@@ -9055,7 +9057,7 @@
       <c r="B345" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="C345" s="2" t="s">
+      <c r="C345" s="5" t="s">
         <v>679</v>
       </c>
       <c r="D345" s="3">
@@ -9072,7 +9074,7 @@
       <c r="B346" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="C346" s="2" t="s">
+      <c r="C346" s="5" t="s">
         <v>681</v>
       </c>
       <c r="D346" s="3">
@@ -9089,7 +9091,7 @@
       <c r="B347" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="C347" s="2" t="s">
+      <c r="C347" s="5" t="s">
         <v>683</v>
       </c>
       <c r="D347" s="3">
@@ -9106,7 +9108,7 @@
       <c r="B348" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="C348" s="2" t="s">
+      <c r="C348" s="5" t="s">
         <v>684</v>
       </c>
       <c r="D348" s="3">
@@ -9123,7 +9125,7 @@
       <c r="B349" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="C349" s="2" t="s">
+      <c r="C349" s="5" t="s">
         <v>685</v>
       </c>
       <c r="D349" s="3">
@@ -9140,7 +9142,7 @@
       <c r="B350" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="C350" s="2" t="s">
+      <c r="C350" s="5" t="s">
         <v>687</v>
       </c>
       <c r="D350" s="3">
@@ -9157,7 +9159,7 @@
       <c r="B351" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="C351" s="2" t="s">
+      <c r="C351" s="5" t="s">
         <v>689</v>
       </c>
       <c r="D351" s="3">
@@ -9174,7 +9176,7 @@
       <c r="B352" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="C352" s="2" t="s">
+      <c r="C352" s="5" t="s">
         <v>691</v>
       </c>
       <c r="D352" s="3">
@@ -9191,7 +9193,7 @@
       <c r="B353" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="C353" s="2" t="s">
+      <c r="C353" s="5" t="s">
         <v>693</v>
       </c>
       <c r="D353" s="3">
@@ -9208,7 +9210,7 @@
       <c r="B354" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="C354" s="2" t="s">
+      <c r="C354" s="5" t="s">
         <v>695</v>
       </c>
       <c r="D354" s="3">
@@ -9225,7 +9227,7 @@
       <c r="B355" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="C355" s="2" t="s">
+      <c r="C355" s="5" t="s">
         <v>697</v>
       </c>
       <c r="D355" s="3">
@@ -9242,7 +9244,7 @@
       <c r="B356" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="C356" s="2" t="s">
+      <c r="C356" s="5" t="s">
         <v>699</v>
       </c>
       <c r="D356" s="3">
@@ -9259,7 +9261,7 @@
       <c r="B357" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="C357" s="2" t="s">
+      <c r="C357" s="5" t="s">
         <v>701</v>
       </c>
       <c r="D357" s="3">
@@ -9276,7 +9278,7 @@
       <c r="B358" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="C358" s="2" t="s">
+      <c r="C358" s="5" t="s">
         <v>703</v>
       </c>
       <c r="D358" s="3">
@@ -9293,7 +9295,7 @@
       <c r="B359" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="C359" s="2" t="s">
+      <c r="C359" s="5" t="s">
         <v>705</v>
       </c>
       <c r="D359" s="3">
@@ -9310,7 +9312,7 @@
       <c r="B360" s="2" t="s">
         <v>195</v>
       </c>
-      <c r="C360" s="2" t="s">
+      <c r="C360" s="5" t="s">
         <v>707</v>
       </c>
       <c r="D360" s="3">
@@ -9327,7 +9329,7 @@
       <c r="B361" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C361" s="2" t="s">
+      <c r="C361" s="5" t="s">
         <v>709</v>
       </c>
       <c r="D361" s="3">
@@ -9344,7 +9346,7 @@
       <c r="B362" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="C362" s="2" t="s">
+      <c r="C362" s="5" t="s">
         <v>710</v>
       </c>
       <c r="D362" s="3">
@@ -9361,7 +9363,7 @@
       <c r="B363" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="C363" s="2" t="s">
+      <c r="C363" s="5" t="s">
         <v>712</v>
       </c>
       <c r="D363" s="3">
@@ -9378,7 +9380,7 @@
       <c r="B364" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="C364" s="2" t="s">
+      <c r="C364" s="5" t="s">
         <v>714</v>
       </c>
       <c r="D364" s="3">
@@ -9395,7 +9397,7 @@
       <c r="B365" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="C365" s="2" t="s">
+      <c r="C365" s="5" t="s">
         <v>716</v>
       </c>
       <c r="D365" s="3">
@@ -9412,7 +9414,7 @@
       <c r="B366" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="C366" s="2" t="s">
+      <c r="C366" s="5" t="s">
         <v>718</v>
       </c>
       <c r="D366" s="3">
@@ -9429,7 +9431,7 @@
       <c r="B367" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="C367" s="2" t="s">
+      <c r="C367" s="5" t="s">
         <v>720</v>
       </c>
       <c r="D367" s="3">
@@ -9446,7 +9448,7 @@
       <c r="B368" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="C368" s="2" t="s">
+      <c r="C368" s="5" t="s">
         <v>722</v>
       </c>
       <c r="D368" s="3">
@@ -9463,7 +9465,7 @@
       <c r="B369" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="C369" s="2" t="s">
+      <c r="C369" s="5" t="s">
         <v>724</v>
       </c>
       <c r="D369" s="3">
@@ -9480,7 +9482,7 @@
       <c r="B370" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="C370" s="2" t="s">
+      <c r="C370" s="5" t="s">
         <v>726</v>
       </c>
       <c r="D370" s="3">
@@ -9497,7 +9499,7 @@
       <c r="B371" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="C371" s="2" t="s">
+      <c r="C371" s="5" t="s">
         <v>728</v>
       </c>
       <c r="D371" s="3">
@@ -9514,7 +9516,7 @@
       <c r="B372" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="C372" s="2" t="s">
+      <c r="C372" s="5" t="s">
         <v>730</v>
       </c>
       <c r="D372" s="3">
@@ -9531,7 +9533,7 @@
       <c r="B373" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="C373" s="2" t="s">
+      <c r="C373" s="5" t="s">
         <v>732</v>
       </c>
       <c r="D373" s="3">
@@ -9548,7 +9550,7 @@
       <c r="B374" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="C374" s="2" t="s">
+      <c r="C374" s="5" t="s">
         <v>734</v>
       </c>
       <c r="D374" s="3">
@@ -9565,7 +9567,7 @@
       <c r="B375" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="C375" s="2" t="s">
+      <c r="C375" s="5" t="s">
         <v>736</v>
       </c>
       <c r="D375" s="3">
@@ -9582,7 +9584,7 @@
       <c r="B376" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="C376" s="2" t="s">
+      <c r="C376" s="5" t="s">
         <v>738</v>
       </c>
       <c r="D376" s="3">
@@ -9599,7 +9601,7 @@
       <c r="B377" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="C377" s="2" t="s">
+      <c r="C377" s="5" t="s">
         <v>740</v>
       </c>
       <c r="D377" s="3">
@@ -9616,7 +9618,7 @@
       <c r="B378" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="C378" s="2" t="s">
+      <c r="C378" s="5" t="s">
         <v>742</v>
       </c>
       <c r="D378" s="3">
@@ -9633,7 +9635,7 @@
       <c r="B379" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="C379" s="2" t="s">
+      <c r="C379" s="5" t="s">
         <v>744</v>
       </c>
       <c r="D379" s="3">
@@ -9650,7 +9652,7 @@
       <c r="B380" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="C380" s="2" t="s">
+      <c r="C380" s="5" t="s">
         <v>746</v>
       </c>
       <c r="D380" s="3">
@@ -9667,7 +9669,7 @@
       <c r="B381" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="C381" s="2" t="s">
+      <c r="C381" s="5" t="s">
         <v>748</v>
       </c>
       <c r="D381" s="3">
@@ -9684,7 +9686,7 @@
       <c r="B382" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="C382" s="2" t="s">
+      <c r="C382" s="5" t="s">
         <v>750</v>
       </c>
       <c r="D382" s="3">
@@ -9701,7 +9703,7 @@
       <c r="B383" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="C383" s="2" t="s">
+      <c r="C383" s="5" t="s">
         <v>752</v>
       </c>
       <c r="D383" s="3">
@@ -9718,7 +9720,7 @@
       <c r="B384" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="C384" s="2" t="s">
+      <c r="C384" s="5" t="s">
         <v>754</v>
       </c>
       <c r="D384" s="3">
@@ -9735,7 +9737,7 @@
       <c r="B385" s="2" t="s">
         <v>195</v>
       </c>
-      <c r="C385" s="2" t="s">
+      <c r="C385" s="5" t="s">
         <v>756</v>
       </c>
       <c r="D385" s="3">
@@ -9752,7 +9754,7 @@
       <c r="B386" s="2" t="s">
         <v>195</v>
       </c>
-      <c r="C386" s="2" t="s">
+      <c r="C386" s="5" t="s">
         <v>758</v>
       </c>
       <c r="D386" s="3">
@@ -9769,7 +9771,7 @@
       <c r="B387" s="2" t="s">
         <v>195</v>
       </c>
-      <c r="C387" s="2" t="s">
+      <c r="C387" s="5" t="s">
         <v>760</v>
       </c>
       <c r="D387" s="3">
@@ -9786,7 +9788,7 @@
       <c r="B388" s="2" t="s">
         <v>195</v>
       </c>
-      <c r="C388" s="2" t="s">
+      <c r="C388" s="5" t="s">
         <v>762</v>
       </c>
       <c r="D388" s="3">
@@ -9803,7 +9805,7 @@
       <c r="B389" s="2" t="s">
         <v>195</v>
       </c>
-      <c r="C389" s="2" t="s">
+      <c r="C389" s="5" t="s">
         <v>764</v>
       </c>
       <c r="D389" s="3">
@@ -9820,7 +9822,7 @@
       <c r="B390" s="2" t="s">
         <v>195</v>
       </c>
-      <c r="C390" s="2" t="s">
+      <c r="C390" s="5" t="s">
         <v>766</v>
       </c>
       <c r="D390" s="3">
@@ -9837,7 +9839,7 @@
       <c r="B391" s="2" t="s">
         <v>195</v>
       </c>
-      <c r="C391" s="2" t="s">
+      <c r="C391" s="5" t="s">
         <v>768</v>
       </c>
       <c r="D391" s="3">
@@ -9854,7 +9856,7 @@
       <c r="B392" s="2" t="s">
         <v>195</v>
       </c>
-      <c r="C392" s="2" t="s">
+      <c r="C392" s="5" t="s">
         <v>770</v>
       </c>
       <c r="D392" s="3">
@@ -9871,7 +9873,7 @@
       <c r="B393" s="2" t="s">
         <v>195</v>
       </c>
-      <c r="C393" s="2" t="s">
+      <c r="C393" s="5" t="s">
         <v>772</v>
       </c>
       <c r="D393" s="3">
@@ -9888,7 +9890,7 @@
       <c r="B394" s="2" t="s">
         <v>195</v>
       </c>
-      <c r="C394" s="2" t="s">
+      <c r="C394" s="5" t="s">
         <v>774</v>
       </c>
       <c r="D394" s="3">
@@ -9905,7 +9907,7 @@
       <c r="B395" s="2" t="s">
         <v>195</v>
       </c>
-      <c r="C395" s="2" t="s">
+      <c r="C395" s="5" t="s">
         <v>776</v>
       </c>
       <c r="D395" s="3">
@@ -9922,7 +9924,7 @@
       <c r="B396" s="2" t="s">
         <v>195</v>
       </c>
-      <c r="C396" s="2" t="s">
+      <c r="C396" s="5" t="s">
         <v>778</v>
       </c>
       <c r="D396" s="3">
@@ -9939,7 +9941,7 @@
       <c r="B397" s="2" t="s">
         <v>195</v>
       </c>
-      <c r="C397" s="2" t="s">
+      <c r="C397" s="5" t="s">
         <v>780</v>
       </c>
       <c r="D397" s="3">
@@ -9956,7 +9958,7 @@
       <c r="B398" s="2" t="s">
         <v>195</v>
       </c>
-      <c r="C398" s="2" t="s">
+      <c r="C398" s="5" t="s">
         <v>782</v>
       </c>
       <c r="D398" s="3">
@@ -9973,7 +9975,7 @@
       <c r="B399" s="2" t="s">
         <v>195</v>
       </c>
-      <c r="C399" s="2" t="s">
+      <c r="C399" s="5" t="s">
         <v>784</v>
       </c>
       <c r="D399" s="3">
@@ -9990,7 +9992,7 @@
       <c r="B400" s="2" t="s">
         <v>195</v>
       </c>
-      <c r="C400" s="2" t="s">
+      <c r="C400" s="5" t="s">
         <v>786</v>
       </c>
       <c r="D400" s="3">
@@ -10007,7 +10009,7 @@
       <c r="B401" s="2" t="s">
         <v>195</v>
       </c>
-      <c r="C401" s="2" t="s">
+      <c r="C401" s="5" t="s">
         <v>788</v>
       </c>
       <c r="D401" s="3">
@@ -10024,7 +10026,7 @@
       <c r="B402" s="2" t="s">
         <v>195</v>
       </c>
-      <c r="C402" s="2" t="s">
+      <c r="C402" s="5" t="s">
         <v>790</v>
       </c>
       <c r="D402" s="3">
@@ -10041,7 +10043,7 @@
       <c r="B403" s="2" t="s">
         <v>195</v>
       </c>
-      <c r="C403" s="2" t="s">
+      <c r="C403" s="5" t="s">
         <v>792</v>
       </c>
       <c r="D403" s="3">
@@ -10058,7 +10060,7 @@
       <c r="B404" s="2" t="s">
         <v>195</v>
       </c>
-      <c r="C404" s="2" t="s">
+      <c r="C404" s="5" t="s">
         <v>794</v>
       </c>
       <c r="D404" s="3">
@@ -10075,7 +10077,7 @@
       <c r="B405" s="2" t="s">
         <v>195</v>
       </c>
-      <c r="C405" s="2" t="s">
+      <c r="C405" s="5" t="s">
         <v>796</v>
       </c>
       <c r="D405" s="3">
@@ -10092,7 +10094,7 @@
       <c r="B406" s="2" t="s">
         <v>195</v>
       </c>
-      <c r="C406" s="2" t="s">
+      <c r="C406" s="5" t="s">
         <v>798</v>
       </c>
       <c r="D406" s="3">
@@ -10109,7 +10111,7 @@
       <c r="B407" s="2" t="s">
         <v>195</v>
       </c>
-      <c r="C407" s="2" t="s">
+      <c r="C407" s="5" t="s">
         <v>800</v>
       </c>
       <c r="D407" s="3">
@@ -10126,7 +10128,7 @@
       <c r="B408" s="2" t="s">
         <v>195</v>
       </c>
-      <c r="C408" s="2" t="s">
+      <c r="C408" s="5" t="s">
         <v>802</v>
       </c>
       <c r="D408" s="3">
@@ -10143,7 +10145,7 @@
       <c r="B409" s="2" t="s">
         <v>195</v>
       </c>
-      <c r="C409" s="2" t="s">
+      <c r="C409" s="5" t="s">
         <v>804</v>
       </c>
       <c r="D409" s="3">
@@ -10160,7 +10162,7 @@
       <c r="B410" s="2" t="s">
         <v>195</v>
       </c>
-      <c r="C410" s="2" t="s">
+      <c r="C410" s="5" t="s">
         <v>806</v>
       </c>
       <c r="D410" s="3">
@@ -10177,7 +10179,7 @@
       <c r="B411" s="2" t="s">
         <v>195</v>
       </c>
-      <c r="C411" s="2" t="s">
+      <c r="C411" s="5" t="s">
         <v>808</v>
       </c>
       <c r="D411" s="3">
@@ -10194,7 +10196,7 @@
       <c r="B412" s="2" t="s">
         <v>195</v>
       </c>
-      <c r="C412" s="2" t="s">
+      <c r="C412" s="5" t="s">
         <v>810</v>
       </c>
       <c r="D412" s="3">
@@ -10211,7 +10213,7 @@
       <c r="B413" s="2" t="s">
         <v>195</v>
       </c>
-      <c r="C413" s="2" t="s">
+      <c r="C413" s="5" t="s">
         <v>812</v>
       </c>
       <c r="D413" s="3">
@@ -10228,7 +10230,7 @@
       <c r="B414" s="2" t="s">
         <v>195</v>
       </c>
-      <c r="C414" s="2" t="s">
+      <c r="C414" s="5" t="s">
         <v>814</v>
       </c>
       <c r="D414" s="3">
@@ -10245,7 +10247,7 @@
       <c r="B415" s="2" t="s">
         <v>195</v>
       </c>
-      <c r="C415" s="2" t="s">
+      <c r="C415" s="5" t="s">
         <v>816</v>
       </c>
       <c r="D415" s="3">
@@ -10262,7 +10264,7 @@
       <c r="B416" s="2" t="s">
         <v>195</v>
       </c>
-      <c r="C416" s="2" t="s">
+      <c r="C416" s="5" t="s">
         <v>818</v>
       </c>
       <c r="D416" s="3">
@@ -10279,7 +10281,7 @@
       <c r="B417" s="2" t="s">
         <v>195</v>
       </c>
-      <c r="C417" s="2" t="s">
+      <c r="C417" s="5" t="s">
         <v>820</v>
       </c>
       <c r="D417" s="3">
@@ -10296,7 +10298,7 @@
       <c r="B418" s="2" t="s">
         <v>195</v>
       </c>
-      <c r="C418" s="2" t="s">
+      <c r="C418" s="5" t="s">
         <v>822</v>
       </c>
       <c r="D418" s="3">
@@ -10313,7 +10315,7 @@
       <c r="B419" s="2" t="s">
         <v>195</v>
       </c>
-      <c r="C419" s="2" t="s">
+      <c r="C419" s="5" t="s">
         <v>824</v>
       </c>
       <c r="D419" s="3">
@@ -10330,7 +10332,7 @@
       <c r="B420" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="C420" s="2" t="s">
+      <c r="C420" s="5" t="s">
         <v>826</v>
       </c>
       <c r="D420" s="3">
@@ -10347,7 +10349,7 @@
       <c r="B421" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="C421" s="2" t="s">
+      <c r="C421" s="5" t="s">
         <v>828</v>
       </c>
       <c r="D421" s="3">
@@ -10364,7 +10366,7 @@
       <c r="B422" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="C422" s="2" t="s">
+      <c r="C422" s="5" t="s">
         <v>830</v>
       </c>
       <c r="D422" s="3">
@@ -10381,7 +10383,7 @@
       <c r="B423" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="C423" s="2" t="s">
+      <c r="C423" s="5" t="s">
         <v>832</v>
       </c>
       <c r="D423" s="3">
@@ -10398,7 +10400,7 @@
       <c r="B424" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="C424" s="2" t="s">
+      <c r="C424" s="5" t="s">
         <v>834</v>
       </c>
       <c r="D424" s="3">
@@ -10415,7 +10417,7 @@
       <c r="B425" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="C425" s="2" t="s">
+      <c r="C425" s="5" t="s">
         <v>836</v>
       </c>
       <c r="D425" s="3">
@@ -10432,7 +10434,7 @@
       <c r="B426" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="C426" s="2" t="s">
+      <c r="C426" s="5" t="s">
         <v>838</v>
       </c>
       <c r="D426" s="3">
@@ -10449,7 +10451,7 @@
       <c r="B427" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="C427" s="2" t="s">
+      <c r="C427" s="5" t="s">
         <v>840</v>
       </c>
       <c r="D427" s="3">
@@ -10466,7 +10468,7 @@
       <c r="B428" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="C428" s="2" t="s">
+      <c r="C428" s="5" t="s">
         <v>842</v>
       </c>
       <c r="D428" s="3">
@@ -10483,7 +10485,7 @@
       <c r="B429" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="C429" s="2" t="s">
+      <c r="C429" s="5" t="s">
         <v>844</v>
       </c>
       <c r="D429" s="3">
@@ -10500,7 +10502,7 @@
       <c r="B430" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="C430" s="2" t="s">
+      <c r="C430" s="5" t="s">
         <v>846</v>
       </c>
       <c r="D430" s="3">
@@ -10517,7 +10519,7 @@
       <c r="B431" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="C431" s="2" t="s">
+      <c r="C431" s="5" t="s">
         <v>848</v>
       </c>
       <c r="D431" s="3">
@@ -10534,7 +10536,7 @@
       <c r="B432" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="C432" s="2" t="s">
+      <c r="C432" s="5" t="s">
         <v>850</v>
       </c>
       <c r="D432" s="3">
@@ -10551,7 +10553,7 @@
       <c r="B433" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="C433" s="2" t="s">
+      <c r="C433" s="5" t="s">
         <v>852</v>
       </c>
       <c r="D433" s="3">
@@ -10568,7 +10570,7 @@
       <c r="B434" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="C434" s="2" t="s">
+      <c r="C434" s="5" t="s">
         <v>854</v>
       </c>
       <c r="D434" s="3">
@@ -10585,7 +10587,7 @@
       <c r="B435" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="C435" s="2" t="s">
+      <c r="C435" s="5" t="s">
         <v>856</v>
       </c>
       <c r="D435" s="3">
@@ -10602,7 +10604,7 @@
       <c r="B436" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="C436" s="2" t="s">
+      <c r="C436" s="5" t="s">
         <v>858</v>
       </c>
       <c r="D436" s="3">
@@ -10619,7 +10621,7 @@
       <c r="B437" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="C437" s="2" t="s">
+      <c r="C437" s="5" t="s">
         <v>860</v>
       </c>
       <c r="D437" s="3">
@@ -10636,7 +10638,7 @@
       <c r="B438" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="C438" s="2" t="s">
+      <c r="C438" s="5" t="s">
         <v>862</v>
       </c>
       <c r="D438" s="3">
@@ -10653,7 +10655,7 @@
       <c r="B439" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="C439" s="2" t="s">
+      <c r="C439" s="5" t="s">
         <v>864</v>
       </c>
       <c r="D439" s="3">
@@ -10670,7 +10672,7 @@
       <c r="B440" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="C440" s="2" t="s">
+      <c r="C440" s="5" t="s">
         <v>866</v>
       </c>
       <c r="D440" s="3">
@@ -10687,7 +10689,7 @@
       <c r="B441" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="C441" s="2" t="s">
+      <c r="C441" s="5" t="s">
         <v>868</v>
       </c>
       <c r="D441" s="3">
@@ -10704,7 +10706,7 @@
       <c r="B442" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="C442" s="2" t="s">
+      <c r="C442" s="5" t="s">
         <v>870</v>
       </c>
       <c r="D442" s="3">
@@ -10721,7 +10723,7 @@
       <c r="B443" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="C443" s="2" t="s">
+      <c r="C443" s="5" t="s">
         <v>872</v>
       </c>
       <c r="D443" s="3">
@@ -10738,7 +10740,7 @@
       <c r="B444" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="C444" s="2" t="s">
+      <c r="C444" s="5" t="s">
         <v>874</v>
       </c>
       <c r="D444" s="3">
@@ -10755,7 +10757,7 @@
       <c r="B445" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="C445" s="2" t="s">
+      <c r="C445" s="5" t="s">
         <v>876</v>
       </c>
       <c r="D445" s="3">
@@ -10772,7 +10774,7 @@
       <c r="B446" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="C446" s="2" t="s">
+      <c r="C446" s="5" t="s">
         <v>878</v>
       </c>
       <c r="D446" s="3">
@@ -10789,7 +10791,7 @@
       <c r="B447" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="C447" s="2" t="s">
+      <c r="C447" s="5" t="s">
         <v>880</v>
       </c>
       <c r="D447" s="3">
@@ -10806,7 +10808,7 @@
       <c r="B448" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="C448" s="2" t="s">
+      <c r="C448" s="5" t="s">
         <v>882</v>
       </c>
       <c r="D448" s="3">
@@ -10823,7 +10825,7 @@
       <c r="B449" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="C449" s="2" t="s">
+      <c r="C449" s="5" t="s">
         <v>884</v>
       </c>
       <c r="D449" s="3">
@@ -10840,7 +10842,7 @@
       <c r="B450" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="C450" s="2" t="s">
+      <c r="C450" s="5" t="s">
         <v>886</v>
       </c>
       <c r="D450" s="3">
@@ -10857,7 +10859,7 @@
       <c r="B451" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="C451" s="2" t="s">
+      <c r="C451" s="5" t="s">
         <v>888</v>
       </c>
       <c r="D451" s="3">
@@ -10874,7 +10876,7 @@
       <c r="B452" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="C452" s="2" t="s">
+      <c r="C452" s="5" t="s">
         <v>890</v>
       </c>
       <c r="D452" s="3">
@@ -10891,7 +10893,7 @@
       <c r="B453" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="C453" s="2" t="s">
+      <c r="C453" s="5" t="s">
         <v>892</v>
       </c>
       <c r="D453" s="3">
@@ -10908,7 +10910,7 @@
       <c r="B454" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="C454" s="2" t="s">
+      <c r="C454" s="5" t="s">
         <v>894</v>
       </c>
       <c r="D454" s="3">
@@ -10925,7 +10927,7 @@
       <c r="B455" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="C455" s="2" t="s">
+      <c r="C455" s="5" t="s">
         <v>896</v>
       </c>
       <c r="D455" s="3">
@@ -10942,7 +10944,7 @@
       <c r="B456" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="C456" s="2" t="s">
+      <c r="C456" s="5" t="s">
         <v>898</v>
       </c>
       <c r="D456" s="3">
@@ -10959,7 +10961,7 @@
       <c r="B457" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="C457" s="2" t="s">
+      <c r="C457" s="5" t="s">
         <v>900</v>
       </c>
       <c r="D457" s="3">
@@ -10976,7 +10978,7 @@
       <c r="B458" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="C458" s="2" t="s">
+      <c r="C458" s="5" t="s">
         <v>902</v>
       </c>
       <c r="D458" s="3">
@@ -10993,7 +10995,7 @@
       <c r="B459" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="C459" s="2" t="s">
+      <c r="C459" s="5" t="s">
         <v>904</v>
       </c>
       <c r="D459" s="3">
@@ -11010,7 +11012,7 @@
       <c r="B460" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="C460" s="2" t="s">
+      <c r="C460" s="5" t="s">
         <v>906</v>
       </c>
       <c r="D460" s="3">
@@ -11027,7 +11029,7 @@
       <c r="B461" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="C461" s="2" t="s">
+      <c r="C461" s="5" t="s">
         <v>908</v>
       </c>
       <c r="D461" s="3">
@@ -11044,7 +11046,7 @@
       <c r="B462" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="C462" s="2" t="s">
+      <c r="C462" s="5" t="s">
         <v>910</v>
       </c>
       <c r="D462" s="3">
@@ -11061,7 +11063,7 @@
       <c r="B463" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="C463" s="2" t="s">
+      <c r="C463" s="5" t="s">
         <v>912</v>
       </c>
       <c r="D463" s="3">
@@ -11078,7 +11080,7 @@
       <c r="B464" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="C464" s="2" t="s">
+      <c r="C464" s="5" t="s">
         <v>914</v>
       </c>
       <c r="D464" s="3">
@@ -11095,7 +11097,7 @@
       <c r="B465" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="C465" s="2" t="s">
+      <c r="C465" s="5" t="s">
         <v>916</v>
       </c>
       <c r="D465" s="3">
@@ -11112,7 +11114,7 @@
       <c r="B466" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="C466" s="2" t="s">
+      <c r="C466" s="5" t="s">
         <v>918</v>
       </c>
       <c r="D466" s="3">

</xml_diff>